<commit_message>
fix: filter TypeScript types/enums from MMDS component counts
- Update mmds-fetcher to only extract actual React/RN components
- Filter out enums like BadgeStatusStatus, ButtonBaseSize, IconName, etc.
- Component must match folder name to be counted
- Exclude common enum suffixes (Size, Variant, Color, Status, Position, etc.)
- Update metrics: Extension 25→21 components, Mobile 34→29 components
- Regenerate 2026-02-27 metrics with accurate component counts
</commit_message>
<xml_diff>
--- a/metrics/extension-component-metrics-2026-02-27.xlsx
+++ b/metrics/extension-component-metrics-2026-02-27.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="185">
   <si>
     <t>Deprecated Component</t>
   </si>
@@ -40,7 +40,7 @@
     <t>ui/components/component-library/text/text.tsx</t>
   </si>
   <si>
-    <t>26.33%</t>
+    <t>26.35%</t>
   </si>
   <si>
     <t>Input</t>
@@ -58,7 +58,7 @@
     <t>ui/components/component-library/icon/icon.tsx</t>
   </si>
   <si>
-    <t>27.52%</t>
+    <t>28.33%</t>
   </si>
   <si>
     <t>Checkbox</t>
@@ -97,7 +97,7 @@
     <t/>
   </si>
   <si>
-    <t>22.57%</t>
+    <t>21.60%</t>
   </si>
   <si>
     <t>ButtonLink</t>
@@ -109,7 +109,7 @@
     <t>TextButton</t>
   </si>
   <si>
-    <t>12.20%</t>
+    <t>18.90%</t>
   </si>
   <si>
     <t>ButtonIcon</t>
@@ -118,7 +118,7 @@
     <t>ui/components/component-library/button-icon/button-icon.tsx</t>
   </si>
   <si>
-    <t>11.30%</t>
+    <t>11.36%</t>
   </si>
   <si>
     <t>ButtonBase</t>
@@ -127,7 +127,7 @@
     <t>ui/components/component-library/button-base/button-base.tsx</t>
   </si>
   <si>
-    <t>62.50%</t>
+    <t>60.53%</t>
   </si>
   <si>
     <t>Box</t>
@@ -136,7 +136,7 @@
     <t>ui/components/component-library/box/box.tsx</t>
   </si>
   <si>
-    <t>30.41%</t>
+    <t>30.80%</t>
   </si>
   <si>
     <t>BadgeWrapper</t>
@@ -148,6 +148,15 @@
     <t>31.58%</t>
   </si>
   <si>
+    <t>AvatarNetwork</t>
+  </si>
+  <si>
+    <t>ui/components/component-library/avatar-network/avatar-network.tsx</t>
+  </si>
+  <si>
+    <t>14.29%</t>
+  </si>
+  <si>
     <t>AvatarToken</t>
   </si>
   <si>
@@ -157,15 +166,6 @@
     <t>27.03%</t>
   </si>
   <si>
-    <t>AvatarNetwork</t>
-  </si>
-  <si>
-    <t>ui/components/component-library/avatar-network/avatar-network.tsx</t>
-  </si>
-  <si>
-    <t>14.29%</t>
-  </si>
-  <si>
     <t>AvatarIcon</t>
   </si>
   <si>
@@ -193,7 +193,7 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>26.91%</t>
+    <t>27.20%</t>
   </si>
   <si>
     <t>Component</t>
@@ -208,364 +208,334 @@
     <t>File Paths</t>
   </si>
   <si>
+    <t>TextFieldSearch</t>
+  </si>
+  <si>
+    <t>ui/components/component-library/text-field-search/deprecated/text-field-search.js</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/swaps/list-with-search/list-with-search.js, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-search/network-list-search.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-search.tsx, repos/metamask-extension/ui/components/app/import-token/token-search/token-search.component.js, repos/metamask-extension/ui/pages/perps/market-list/components/search-input/search-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-filter-input/recipient-filter-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-filter-input/asset-filter-input.tsx</t>
+  </si>
+  <si>
     <t>Textarea</t>
   </si>
   <si>
+    <t>repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/components/ui/textarea/textarea.stories.js, repos/metamask-extension/ui/components/ui/textarea/textarea.stories.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx</t>
+  </si>
+  <si>
+    <t>TextField</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/formatted-counter.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/confirm-add-suggested-token/confirm-add-suggested-token.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/notification-page/notification-page.js, repos/metamask-extension/ui/pages/swaps/notification-page/notification-page.js, repos/metamask-extension/ui/pages/swaps/list-with-search/list-with-search.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/swaps/loading-swaps-quotes/loading-swaps-quotes.js, repos/metamask-extension/ui/pages/swaps/loading-swaps-quotes/loading-swaps-quotes.js, repos/metamask-extension/ui/pages/swaps/fee-card/fee-card.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/url-display-box.tsx, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-message.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-detail-row.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-description.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-description.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-activity-item-tx-segments.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-tx-declined-message.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-no-fee-message.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-info-text.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-button.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle/smart-contract-account-toggle.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu-items/multichain-account-menu-items.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-srp-row/account-show-srp-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/token-balance/token-balance.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/origin-pill/origin-pill.tsx, repos/metamask-extension/ui/components/ui/numeric-input/numeric-input.component.js, repos/metamask-extension/ui/components/ui/metafox-logo/metafox-logo.stories.js, repos/metamask-extension/ui/components/ui/logo/logo.stories.js, repos/metamask-extension/ui/components/ui/icon-button/icon-button.tsx, repos/metamask-extension/ui/components/ui/icon-button/icon-button.tsx, repos/metamask-extension/ui/components/ui/icon/icon.stories.js, repos/metamask-extension/ui/components/ui/icon/icon.stories.js, repos/metamask-extension/ui/components/ui/icon/icon.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/export-text-container/export-text-container.component.js, repos/metamask-extension/ui/components/ui/delineator/delineator.stories.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.stories.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.stories.tsx, repos/metamask-extension/ui/components/ui/disclosure/disclosure.js, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/confusable/confusable.component.js, repos/metamask-extension/ui/components/ui/confusable/confusable.component.js, repos/metamask-extension/ui/components/ui/chip/chip.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.js, repos/metamask-extension/ui/components/ui/actionable-message/actionable-message.stories.js, repos/metamask-extension/ui/components/ui/actionable-message/actionable-message.stories.js, repos/metamask-extension/ui/components/ui/actionable-message/actionable-message.stories.js, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-text/notification-list-item-text.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-text/notification-list-item-text.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-title/notification-detail-title.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-title/notification-detail-title.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-info/notification-detail-info.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-info/notification-detail-info.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-collection/notification-detail-collection.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-address/notification-detail-address.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-asset/notification-detail-asset.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/menu-items/view-explorer-menu-item.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/menu-items/account-details-menu-item.js, repos/metamask-extension/ui/components/multichain/import-account/json.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-unlocked-content.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/selected-account/selected-account.component.js, repos/metamask-extension/ui/components/app/selected-account/selected-account.component.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.stories.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.stories.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/permissions-connect-footer/permissions-connect-footer.component.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/name/name.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/snap-account-success-message/SnapAccountSuccessMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/snap-account-error-message/SnapAccountErrorMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-contract-with-logo/smart-contract-with-logo.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/asset-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/amount-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/confirmations/components/contract-token-values/contract-token-values.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/asset/components/chart/chart-tooltip.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card-empty/stack-card-empty.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card-empty/stack-card-empty.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card/stack-card.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card/stack-card.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-update-alert/snap-update-alert.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-markdown/snap-ui-markdown.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-button/snap-ui-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address/snap-ui-address.tsx, repos/metamask-extension/ui/components/app/snaps/snap-settings-page/snap-settings-renderer.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-page/snap-home-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-pill/snap-authorship-pill.tsx, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/name/name-details/shortened-name.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-display.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/formatted-value.tsx, repos/metamask-extension/ui/components/app/modals/transaction-confirmed/transaction-confirmed.component.js, repos/metamask-extension/ui/components/app/modals/transaction-confirmed/transaction-confirmed.component.js, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/convert-token-to-nft-modal/convert-token-to-nft-modal.js, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-address/detected-token-address.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/alerts/unconnected-account-alert/unconnected-account-alert.js, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/send-utils/send-content/add-recipient/domain-input.component.js, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/ShieldCoverageAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/NonContractAddressAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/NonContractAddressAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/NonContractAddressAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/PendingTransactionAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/AccountTypeMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-list/recipient-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-list/recipient-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/total-row/total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/required-tokens-row/required-tokens-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/bridge-fee-row/bridge-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/bridge-fee-row/bridge-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/bridge-time-row/bridge-time-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/network-statistics/network-statistics.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/network-statistics/network-statistics.js, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/developer/confirmations-developer-options/confirmations-developer-options.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/confirmations-developer-options/confirmations-developer-options.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/wallet-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/dapp-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-agreement.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-gas-limit/advanced-gas-fee-gas-limit.js, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-row/transaction-details-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-status-row/transaction-details-status-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-total-row/transaction-details-total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-network-fee-row/transaction-details-network-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-paid-with-row/transaction-details-paid-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-date-row/transaction-details-date-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-date-row/transaction-details-date-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-account-row/transaction-details-account-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-bridge-fee-row/transaction-details-bridge-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-hero/transaction-details-hero.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-change/percentage-change.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-and-amount-change/percentage-and-amount-change.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-and-amount-change/percentage-and-amount-change.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/value-double.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/value-double.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/text.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/date.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/address.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/sort-control/sort-control.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/asset-title.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/snaps/snaps-section/snap-insight.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/snaps/snaps-section/snap-insight.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-footer-coverage-indicator.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/network-row/network-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/selected-gas-fee-token/selected-gas-fee-token.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/siwe-sign/siwe-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/decoded-simulation/decoded-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx</t>
+  </si>
+  <si>
+    <t>Tag</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/notifications/NewFeatureTag.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/useGlobalMenuSections.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/nested-transaction-tag/nested-transaction-tag.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/account-type-label/account-type-label.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-title.tsx</t>
+  </si>
+  <si>
+    <t>SensitiveText</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.tsx, repos/metamask-extension/ui/components/ui/currency-display/currency-display.component.js, repos/metamask-extension/ui/components/ui/currency-display/currency-display.component.js, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance/account-group-balance.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-secondary-display.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-protocol-cell.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-grouped-symbol-cell.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-primary-display.tsx</t>
+  </si>
+  <si>
+    <t>SuccessPill</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/transaction-breakdown/transaction-breakdown.component.js, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx</t>
+  </si>
+  <si>
+    <t>Skeleton</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsPointsBalance.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-loading.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-start-trade-cta-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-start-trade-cta-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-section-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance/account-group-balance.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/loading-skeleton.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/loading-skeleton.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/loading-skeleton.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-secondary-display.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-primary-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/alert-row/alert-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/token-amount-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx</t>
+  </si>
+  <si>
+    <t>SelectButton</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/selected-asset-button.tsx</t>
+  </si>
+  <si>
+    <t>PopoverHeader</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx</t>
+  </si>
+  <si>
+    <t>PickerNetwork</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/components/multichain/app-header/app-header-locked-content.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx</t>
+  </si>
+  <si>
+    <t>ModalOverlay</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+  </si>
+  <si>
+    <t>Popover</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-filter-menu/index.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/index.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/network-picker.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx</t>
+  </si>
+  <si>
+    <t>ModalHeader</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/network-manager/network-tabs.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+  </si>
+  <si>
+    <t>ModalFocus</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js</t>
+  </si>
+  <si>
+    <t>ModalContent</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+  </si>
+  <si>
+    <t>ModalFooter</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+  </si>
+  <si>
+    <t>ModalBody</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-tabs.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+  </si>
+  <si>
+    <t>Modal</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+  </si>
+  <si>
+    <t>LottieAnimation</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-date-time-picker/snap-ui-date-time-picker.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-dropdown/snap-ui-dropdown.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/index.tsx</t>
+  </si>
+  <si>
+    <t>HelpText</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-date-time-picker/snap-ui-date-time-picker.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-dropdown/snap-ui-dropdown.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/confirm-decrypt-message/confirm-decrypt-message.component.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/pages/swaps/notification-page/notification-page.js, repos/metamask-extension/ui/pages/swaps/selected-token/selected-token.js, repos/metamask-extension/ui/pages/swaps/exchange-rate-display/exchange-rate-display.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/settings/settings-search-list/settings-search-list.js, repos/metamask-extension/ui/pages/settings/settings-search-list/settings-search-list.js, repos/metamask-extension/ui/pages/settings/settings-search/settings-search.js, repos/metamask-extension/ui/pages/settings/settings-search/settings-search.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-list-tab.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/asset-breadcrumb.js, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/step-progress-bar-item.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu-items/multichain-account-menu-items.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/sender-to-recipient/sender-to-recipient.component.js, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/icon-button/icon-button.stories.tsx, repos/metamask-extension/ui/components/ui/icon-button/icon-button.stories.tsx, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/dropdown/dropdown.js, repos/metamask-extension/ui/components/ui/disclosure/disclosure.js, repos/metamask-extension/ui/components/ui/disclosure/disclosure.js, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.js, repos/metamask-extension/ui/components/app/selected-account/selected-account.component.js, repos/metamask-extension/ui/components/app/rewards/RewardsErrorToast.tsx, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/home-notification/home-notification.component.js, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.stories.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail/transaction-detail.stories.js, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/app/transaction-activity-log/transaction-activity-log-icon/transaction-activity-log-icon.component.js, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-markdown/snap-ui-markdown.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-icon/snap-ui-icon.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-footer-button/snap-ui-footer-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-button/snap-ui-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/name/name-details/name-display.tsx, repos/metamask-extension/ui/components/app/modals/transaction-confirmed/transaction-confirmed.component.js, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/alerts/unconnected-account-alert/unconnected-account-alert.js, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-status-icon/transaction-status-icon.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/selected-gas-fee-token/selected-gas-fee-token.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx</t>
+  </si>
+  <si>
+    <t>FormTextField</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/ui/form-combo-field/form-combo-field.tsx, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/private-key.js, repos/metamask-extension/ui/components/multichain/import-account/json.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-price-input/gas-price-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-input/gas-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-input/snap-ui-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-input/snap-ui-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx</t>
+  </si>
+  <si>
+    <t>HeaderBase</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/notification-details/notification-details-header/notification-details-header.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.tsx</t>
+  </si>
+  <si>
+    <t>FileUploader</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx</t>
+  </si>
+  <si>
+    <t>Container</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/bridge/layout/row.tsx, repos/metamask-extension/ui/pages/bridge/layout/column.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.stories.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.stories.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/create-new-vault/create-new-vault.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-defaults/advanced-gas-fee-defaults.js</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-explorer-links.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-explorer-links.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/ui/export-text-container/export-text-container.component.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/bottom-buttons.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-section.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-accounts-page/multichain-edit-accounts-page.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/fee-card/fee-card.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-private-key-list-page/multichain-account-private-key-list-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-tx-declined-message.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-button.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/import-account/json.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-overview.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permissions-connect-footer/permissions-connect-footer.component.js, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/update-snap-permission-list/update-snap-permission-list.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-markdown/snap-ui-markdown.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-address/detected-token-address.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/ShieldCoverageAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/PendingTransactionAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/AccountTypeMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-agreement.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/nft-default-image.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications/notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/confirm-decrypt-message/confirm-decrypt-message.component.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/bridge/index.tsx, repos/metamask-extension/ui/pages/bridge/index.tsx, repos/metamask-extension/ui/pages/snaps/snap-view/snap-view.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/redirect-url-icon.tsx, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-header/notification-details-header.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-options.js, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-srp-row/account-show-srp-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/nickname-popover/nickname-popover.component.js, repos/metamask-extension/ui/components/ui/form-combo-field/form-combo-field.tsx, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/callout/callout.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-unlocked-content.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/contract-token-values/contract-token-values.js, repos/metamask-extension/ui/pages/confirmations/components/contract-token-values/contract-token-values.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-accounts-page/multichain-edit-accounts-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card/stack-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/new-account-modal/new-account-modal.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/edit-approval-permission/edit-approval-permission.component.js, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-options/connected-accounts-list-options.component.js, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/send-utils/send-content/add-recipient/domain-input.component.js, repos/metamask-extension/ui/pages/confirmations/send-utils/send-content/add-recipient/domain-input.component.js, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/scroll-to-bottom/scroll-to-bottom.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/wallet-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/advanced-details-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/block-explorer-link/block-explorer-link.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/index.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/text.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/copy-icon.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.stories.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-secondary-display.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-list-tab.component.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/bottom-buttons.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.stories.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/components/ui/icon-button/icon-button.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-copy-button/notification-detail-copy-button.tsx, repos/metamask-extension/ui/components/multichain/network-filter-menu/index.tsx, repos/metamask-extension/ui/components/multichain/address-copy-button/address-copy-button.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/import-control/import-control.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-read-all-button.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/connected-sites/connected-sites.component.js, repos/metamask-extension/ui/pages/connected-sites/connected-sites.component.js, repos/metamask-extension/ui/pages/confirm-add-suggested-token/confirm-add-suggested-token.js, repos/metamask-extension/ui/pages/swaps/select-quote-popover/select-quote-popover.js, repos/metamask-extension/ui/pages/swaps/select-quote-popover/select-quote-popover.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.stories.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.stories.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.stories.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/account-list.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/account-list.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures-cancel-button.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-button.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.stories.tsx, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/multichain/notification-detail-button/notification-detail-button.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.stories.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.stories.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/home-notification/home-notification.component.js, repos/metamask-extension/ui/components/app/home-notification/home-notification.component.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.stories.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/create-new-vault/create-new-vault.js, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.stories.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.stories.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-icon/edit-gas-fee-icon.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/ui/page-container/page-container-footer/page-container-footer.component.js, repos/metamask-extension/ui/components/ui/page-container/page-container-footer/page-container-footer.component.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.stories.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.stories.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-footer-button/snap-ui-footer-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/new-account-modal/new-account-modal.component.js, repos/metamask-extension/ui/components/app/modals/new-account-modal/new-account-modal.component.js, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.stories.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hide-token-confirmation-modal/hide-token-confirmation-modal.js, repos/metamask-extension/ui/components/app/modals/hide-token-confirmation-modal/hide-token-confirmation-modal.js, repos/metamask-extension/ui/components/app/flask/experimental-area/experimental-area.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-selection-popover/detected-token-selection-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-selection-popover/detected-token-selection-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/alerts/unconnected-account-alert/unconnected-account-alert.js, repos/metamask-extension/ui/components/app/alerts/invalid-custom-network-alert/invalid-custom-network-alert.js, repos/metamask-extension/ui/components/app/alerts/invalid-custom-network-alert/invalid-custom-network-alert.js, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-footer/confirmation-footer.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-footer/confirmation-footer.js, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount-recipient/amount-recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-save/advanced-gas-fee-save.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-gas-limit/advanced-gas-fee-gas-limit.js, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-icon/edit-gas-icon-button.tsx</t>
+  </si>
+  <si>
+    <t>BannerTip</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/snap-account-redirect.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/snap-account-redirect.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/permissions-connect/permissions-connect.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/permissions-connect/permissions-connect.stories.js, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-flow.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-flow.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.stories.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.stories.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.stories.tsx, repos/metamask-extension/ui/pages/notifications/notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-read-all-button.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-item.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-item.stories.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/url-display-box.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-message.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snaps/snap-view/snap-view.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-animation.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-toggle-row-component.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/create-password/create-password.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-body/notification-details-body.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-footer/notification-details-footer.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-footer/notification-details-footer.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/confirmation.js, repos/metamask-extension/ui/pages/confirmations/confirmation/confirmation.js, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/segment.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/segment.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-detail-row.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/hollow-circle.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/pulsing-circle.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/pulsing-circle.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/segment.stories.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-list.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-description.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-activity-item-tx-segments.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-activity-item-tx-segments.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-explorer-links.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-list.stories.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-list.stories.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle/smart-contract-account-toggle.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/multichain-site-cell.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu-items/multichain-account-menu-items.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-srp-row/account-show-srp-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/origin-pill/origin-pill.tsx, repos/metamask-extension/ui/components/ui/metafox-logo/metafox-logo.component.js, repos/metamask-extension/ui/components/ui/logo/logo.stories.js, repos/metamask-extension/ui/components/ui/loading-screen/loading-screen.component.js, repos/metamask-extension/ui/components/ui/loading-screen/loading-screen.component.js, repos/metamask-extension/ui/components/ui/loading-screen/loading-screen.component.js, repos/metamask-extension/ui/components/ui/loading-indicator/loading-indicator.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/export-text-container/export-text-container.component.js, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/currency-display/currency-display.component.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-title/notification-detail-title.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-nft/notification-detail-nft.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-nft/notification-detail-nft.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-copy-button/notification-detail-copy-button.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-collection/notification-detail-collection.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-tabs.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-filter-menu/index.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/bottom-buttons.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/carousel/carousel.tsx, repos/metamask-extension/ui/components/multichain/carousel/carousel.tsx, repos/metamask-extension/ui/components/multichain/app-header/multichain-meta-fox-logo.js, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header.js, repos/metamask-extension/ui/components/multichain/app-header/app-header-container.tsx, repos/metamask-extension/ui/components/multichain/badge-status/badge-status.tsx, repos/metamask-extension/ui/components/multichain/badge-status/badge-status.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.stories.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.stories.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.stories.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-copy-button/address-copy-button.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/account-overview/account-overview-unknown.tsx, repos/metamask-extension/ui/components/multichain/account-overview/account-overview-unknown.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/app/wallet-overview/coin-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list-item-details/transaction-list-item-details.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/smart-transaction-list-item.component.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permissions-connect-permission-list/permissions-connect-permission-list.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permissions-connect-footer/permissions-connect-footer.component.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container.component.js, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/name/name.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/currency-input/currency-input.js, repos/metamask-extension/ui/components/app/currency-input/currency-input.js, repos/metamask-extension/ui/components/app/currency-input/currency-input.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/stories/util.js, repos/metamask-extension/ui/pages/confirmations/confirmation/stories/util.js, repos/metamask-extension/ui/pages/confirmations/confirmation/stories/util.js, repos/metamask-extension/ui/pages/confirmations/components/smart-contract-with-logo/smart-contract-with-logo.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/asset-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/asset-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/amount-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/asset/components/chart/chart-tooltip.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-empty-state.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-loading.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-search/network-list-search.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-search.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/update-snap-permission-list/update-snap-permission-list.js, repos/metamask-extension/ui/components/app/snaps/update-snap-permission-list/update-snap-permission-list.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-renderer/snap-ui-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-renderer/snap-ui-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address/snap-ui-address.tsx, repos/metamask-extension/ui/components/app/snaps/snap-settings-page/snap-settings-renderer.tsx, repos/metamask-extension/ui/components/app/snaps/snap-settings-page/snap-settings-renderer.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-dropdown/snap-ui-dropdown.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-form/snap-ui-form.tsx, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-page/snap-home-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-home-page/snap-home-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-pill/snap-authorship-pill.tsx, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hide-token-confirmation-modal/hide-token-confirmation-modal.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/index.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-details/detected-token-details.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-details/detected-token-details.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-address/detected-token-address.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.stories.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/assets/defi-list/defi-list.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance/account-group-balance.tsx, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/components/transactions/nested-transaction-tag/nested-transaction-tag.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-filter-input/recipient-filter-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-filter-input/asset-filter-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount-recipient/amount-recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount-recipient/amount-recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/total-row/total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/total-row/total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/required-tokens-row/required-tokens-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/scroll-to-bottom/scroll-to-bottom.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/scroll-to-bottom/scroll-to-bottom.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/dataTree.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/wallet-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/advanced-details-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/dapp-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/dapp-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-agreement.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/blockaid-loading-indicator/blockaid-loading-indicator.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-defaults/advanced-gas-fee-defaults.js, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-row/transaction-details-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-status-row/transaction-details-status-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-paid-with-row/transaction-details-paid-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-date-row/transaction-details-date-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-hero/transaction-details-hero.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-change/percentage-change.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-and-amount-change/percentage-and-amount-change.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/value-double.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/index.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/text.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/section.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/currency.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/date.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/address.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/address.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/nft-default-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/sort-control/sort-control.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/sort-control/sort-control.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/typed-sign-data/typedSignData.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/typed-sign-data/typedSignData.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/snaps/snaps-section/snaps-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/typed-sign-data-v1/typedSignDataV1.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/typed-sign-data-v1/typedSignDataV1.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/nft-token-transfer/nft-token-transfer.stories.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/token-transfer.stories.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-footer-coverage-indicator.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-footer-coverage-indicator.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/native-transfer/native-transfer.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/content/content.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/alert-row/alert-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/alert-row/alert-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/static-simulation/static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/transaction-data/transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/transaction-data/transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/transaction-data/transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/transaction-data/transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/network-row/network-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/selected-gas-fee-token/selected-gas-fee-token.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-details/gas-fees-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-toast/gas-fee-token-toast.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-icon/gas-fee-token-icon.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-icon/gas-fee-token-icon.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/confirm-loader/confirm-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/batched-approval-function/batched-approval-function.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/siwe-sign/siwe-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/revoke-set-approval-for-all-static-simulation/revoke-set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/revoke-set-approval-for-all-static-simulation/revoke-set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/revoke-set-approval-for-all-static-simulation/revoke-set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/revoke-set-approval-for-all-static-simulation/revoke-set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/batch/nested-transaction-data/nested-transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/revoke-static-simulation/revoke-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/revoke-static-simulation/revoke-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/revoke-static-simulation/revoke-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/revoke-static-simulation/revoke-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/permit-simulation/permit-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/permit-simulation/permit-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx</t>
+  </si>
+  <si>
+    <t>BannerBase</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx</t>
+  </si>
+  <si>
+    <t>BannerAlert</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/confirm-add-suggested-token/confirm-add-suggested-token.js, repos/metamask-extension/ui/pages/confirm-add-suggested-token/confirm-add-suggested-token.js, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-private-key-list-page/multichain-account-private-key-list-page.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/menu/menu.stories.js, repos/metamask-extension/ui/components/ui/icon-border/icon-border.stories.js, repos/metamask-extension/ui/components/ui/icon-with-fallback/icon-with-fallback.stories.js, repos/metamask-extension/ui/components/ui/chip/chip.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/detected-token-banner/detected-token-banner.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/contact-list/contact-list.component.js, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-error-banner.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-error-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-error-message/simulation-error-message.js, repos/metamask-extension/ui/pages/confirmations/components/simulation-error-message/simulation-error-message.js, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/components/app/snaps/snap-update-alert/snap-update-alert.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-banner/snap-ui-banner.tsx, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-detection-notice-import-nfts/nfts-detection-notice-import-nfts.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-detection-notice-nfts-tab/nfts-detection-notice-nfts-tab.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-collection/notification-detail-collection.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-asset/notification-detail-asset.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/multichain/badge-status/badge-status.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/smart-transaction-list-item.component.js, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/token-icon/token-icon.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-details/detected-token-details.js, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/asset-cell-badge.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/smart-transaction-list-item.component.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/token-icon/token-icon.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/asset-pill.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-details/detected-token-details.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/asset-cell-badge.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/network-row/network-row.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-collection/notification-detail-collection.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-asset/notification-detail-asset.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-asset/notification-detail-asset.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-asset/notification-detail-asset.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/pages/confirmations/components/token-icon/token-icon.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-details/detected-token-details.js, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/asset-cell-badge.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-icon/gas-fee-token-icon.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-info/notification-detail-info.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/app/transaction-icon/transaction-icon.js, repos/metamask-extension/ui/components/app/transaction-icon/transaction-icon.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/components/ui/origin-pill/origin-pill.tsx, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-sites-list.component.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-icon/snap-icon.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-icon/snap-icon.tsx</t>
+  </si>
+  <si>
+    <t>AvatarAccount</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/components/ui/identicon/identicon.component.js, repos/metamask-extension/ui/components/multichain/toast/toast.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/app/preferred-avatar/preferred-avatar.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx</t>
+  </si>
+  <si>
+    <t>AvatarGroup</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/network-picker.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/permission-item.tsx, repos/metamask-extension/ui/components/app/chain-badge/chain-badge.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/selected-asset-button.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/components/app/perps/perps-token-logo/perps-token-logo.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/selected-asset-button.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/native-amount-row.tsx</t>
+  </si>
+  <si>
+    <t>BadgeCount</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx</t>
+  </si>
+  <si>
+    <t>BadgeIcon</t>
+  </si>
+  <si>
+    <t>BadgeNetwork</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx, repos/metamask-extension/ui/components/app/chain-badge/chain-badge.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/selected-asset-button.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/settings/settings-toggle-item.tsx, repos/metamask-extension/ui/pages/settings/settings-toggle-item.tsx, repos/metamask-extension/ui/pages/rewards/index.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/create-account/create-account.component.js, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/shield-banner-animation.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/shield-banner-animation.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/experimental-tab/experimental-tab.tsx, repos/metamask-extension/ui/pages/settings/backup-and-sync-tab/backup-and-sync-tab.tsx, repos/metamask-extension/ui/pages/settings/backup-and-sync-tab/backup-and-sync-tab.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/metamask-wordmark-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/metamask-wordmark-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/fox-appear-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/fox-appear-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/setting.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/setting.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/setting.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/wallet-ready-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/wallet-ready-animation.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-private-key-list-page/multichain-account-private-key-list-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/smart-account-page/smart-account-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-address-list-page/multichain-account-address-list-page.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-aggregated-list-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-aggregated-list-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-aggregated-list-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-network-group-with-default-address/multichain-account-network-group-with-default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-network-group/multichain-account-network-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/ui/tab-empty-state/tab-empty-state.tsx, repos/metamask-extension/ui/components/ui/tabs/tabs.tsx, repos/metamask-extension/ui/components/ui/tabs/tabs.tsx, repos/metamask-extension/ui/components/ui/tabs/tabs.tsx, repos/metamask-extension/ui/components/multichain/menu-items/discover-menu-item.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/useGlobalMenuSections.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/useGlobalMenuSections.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/permission-item.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/permission-item.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-unlocked-content.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list-item.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-illustration-animation.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-illustration-animation.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsBadge.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsBadge.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsBadge.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorToast.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/balance-empty-state/balance-empty-state.tsx, repos/metamask-extension/ui/components/app/balance-empty-state/balance-empty-state.tsx, repos/metamask-extension/ui/components/app/balance-empty-state/balance-empty-state.tsx, repos/metamask-extension/ui/components/app/api-error-handler/api-error-handler.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row-container.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/crypto-account-display.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-price-input/gas-price-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-input/gas-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-date-time-picker/snap-ui-date-time-picker.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/ProgressIndicator.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/ProgressIndicator.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialAnimation.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialAnimation.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/TutorialFooter.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/ProgressIndicator.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/ProgressIndicator.tsx, repos/metamask-extension/ui/components/app/perps/start-trade-cta/start-trade-cta.tsx, repos/metamask-extension/ui/components/app/perps/start-trade-cta/start-trade-cta.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-start-trade-cta-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-section-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-section-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-section-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-candlestick-chart/perps-candlestick-chart.tsx, repos/metamask-extension/ui/components/app/perps/perps-empty-state/perps-empty-state.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/quote-swap-simulation-details/quote-swap-simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/quote-swap-simulation-details/quote-swap-simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/quote-swap-simulation-details/quote-swap-simulation-details.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/review-permissions/review-gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/token-transfer/token-transfer-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/CloseAnytimeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/CloseAnytimeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WatchLiquidationStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WatchLiquidationStep.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ChooseLeverageStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ChooseLeverageStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ReadyToTradeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ReadyToTradeStep.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-title.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/estimated-changes.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-icon-animation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-icon-animation.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/direction-tabs/direction-tabs.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/token-amount-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/native-amount-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/date-and-time-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/quote-transaction-data/quoted-transaction-data.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.stories.tsx, repos/metamask-extension/ui/components/ui/tab-empty-state/tab-empty-state.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list-item-details/transaction-list-item-details.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/cancel-button/cancel-button.js, repos/metamask-extension/ui/components/app/balance-empty-state/balance-empty-state.tsx, repos/metamask-extension/ui/components/app/api-error-handler/api-error-handler.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/reactivate-button.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/TutorialFooter.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/TutorialFooter.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/start-trade-cta/start-trade-cta.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/direction-tabs/direction-tabs.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/direction-tabs/direction-tabs.tsx</t>
+  </si>
+  <si>
+    <t>ButtonHero</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-private-key-list-page/multichain-account-private-key-list-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/smart-account-page/smart-account-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/add-wallet-page/add-wallet-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-address-list-page/multichain-account-address-list-page.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/review-permissions/review-gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/token-transfer/token-transfer-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-aggregated-list-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-network-group-with-default-address/multichain-account-network-group-with-default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-unlocked-content.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsBadge.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsBadge.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/AddRewardsAccount.tsx, repos/metamask-extension/ui/components/app/rewards/AddRewardsAccount.tsx, repos/metamask-extension/ui/components/app/musd/claim-bonus-badge.tsx, repos/metamask-extension/ui/components/app/api-error-handler/api-error-handler.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/crypto-account-display.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/perps/start-trade-cta/start-trade-cta.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-empty-state/perps-empty-state.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/settings/settings-toggle-item.tsx, repos/metamask-extension/ui/pages/settings/settings-toggle-item.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-order-entry-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/migrate-to-split-state-test.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/setting.tsx, repos/metamask-extension/ui/pages/multichain-accounts/add-wallet-page/add-wallet-page.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-aggregated-list-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-aggregated-list-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-network-group-with-default-address/multichain-account-network-group-with-default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/ui/tab-empty-state/tab-empty-state.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/permission-item.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/permission-item.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/non-evm-activity-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list-item.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsBadge.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/musd/claim-bonus-badge.tsx, repos/metamask-extension/ui/components/app/musd/claim-bonus-badge.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/balance-empty-state/balance-empty-state.tsx, repos/metamask-extension/ui/components/app/balance-empty-state/balance-empty-state.tsx, repos/metamask-extension/ui/components/app/api-error-handler/api-error-handler.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/crypto-account-display.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-price-input/gas-price-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/components/ui/tabs/tab/tab.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/start-trade-cta/start-trade-cta.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/quote-swap-simulation-details/quote-swap-simulation-details.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/lazy-asset-list.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/review-permissions/review-gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/CloseAnytimeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/CloseAnytimeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WatchLiquidationStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WatchLiquidationStep.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ChooseLeverageStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ChooseLeverageStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ReadyToTradeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ReadyToTradeStep.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/direction-tabs/direction-tabs.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/direction-tabs/direction-tabs.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/native-token-periodic-details.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/native-amount-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/erc20-token-periodic-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/date-and-time-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/date-and-time-row.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/app/rewards/AddRewardsAccount.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx</t>
+  </si>
+  <si>
+    <t>Path</t>
+  </si>
+  <si>
     <t>ui/components/component-library/textarea/textarea.tsx</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/components/ui/textarea/textarea.stories.js, repos/metamask-extension/ui/components/ui/textarea/textarea.stories.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx</t>
-  </si>
-  <si>
-    <t>TextFieldSearch</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/swaps/list-with-search/list-with-search.js, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-search/network-list-search.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-search.tsx, repos/metamask-extension/ui/components/app/import-token/token-search/token-search.component.js, repos/metamask-extension/ui/pages/perps/market-list/components/search-input/search-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-filter-input/recipient-filter-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-filter-input/asset-filter-input.tsx</t>
-  </si>
-  <si>
-    <t>TextField</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/formatted-counter.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/confirm-add-suggested-token/confirm-add-suggested-token.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/loading-swaps-quotes/loading-swaps-quotes.js, repos/metamask-extension/ui/pages/swaps/loading-swaps-quotes/loading-swaps-quotes.js, repos/metamask-extension/ui/pages/swaps/notification-page/notification-page.js, repos/metamask-extension/ui/pages/swaps/notification-page/notification-page.js, repos/metamask-extension/ui/pages/swaps/list-with-search/list-with-search.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/swaps/fee-card/fee-card.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/url-display-box.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-message.tsx, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-detail-row.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-description.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-description.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-activity-item-tx-segments.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-tx-declined-message.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-no-fee-message.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-button.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-info-text.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/components/ui/token-balance/token-balance.js, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/numeric-input/numeric-input.component.js, repos/metamask-extension/ui/components/ui/origin-pill/origin-pill.tsx, repos/metamask-extension/ui/components/ui/metafox-logo/metafox-logo.stories.js, repos/metamask-extension/ui/components/ui/logo/logo.stories.js, repos/metamask-extension/ui/components/ui/icon-button/icon-button.tsx, repos/metamask-extension/ui/components/ui/icon-button/icon-button.tsx, repos/metamask-extension/ui/components/ui/icon/icon.stories.js, repos/metamask-extension/ui/components/ui/icon/icon.stories.js, repos/metamask-extension/ui/components/ui/icon/icon.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/export-text-container/export-text-container.component.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/disclosure/disclosure.js, repos/metamask-extension/ui/components/ui/delineator/delineator.stories.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.stories.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.stories.tsx, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/confusable/confusable.component.js, repos/metamask-extension/ui/components/ui/confusable/confusable.component.js, repos/metamask-extension/ui/components/ui/chip/chip.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/actionable-message/actionable-message.stories.js, repos/metamask-extension/ui/components/ui/actionable-message/actionable-message.stories.js, repos/metamask-extension/ui/components/ui/actionable-message/actionable-message.stories.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle/smart-contract-account-toggle.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu-items/multichain-account-menu-items.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-srp-row/account-show-srp-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-text/notification-list-item-text.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-text/notification-list-item-text.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-title/notification-detail-title.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-title/notification-detail-title.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-info/notification-detail-info.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-info/notification-detail-info.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-collection/notification-detail-collection.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-asset/notification-detail-asset.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-address/notification-detail-address.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/menu-items/view-explorer-menu-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/menu-items/account-details-menu-item.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/json.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-unlocked-content.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/selected-account/selected-account.component.js, repos/metamask-extension/ui/components/app/selected-account/selected-account.component.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permissions-connect-footer/permissions-connect-footer.component.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.stories.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.stories.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/name/name.tsx, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/snap-account-success-message/SnapAccountSuccessMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/snap-account-error-message/SnapAccountErrorMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-contract-with-logo/smart-contract-with-logo.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/asset-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/amount-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/contract-token-values/contract-token-values.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/pages/asset/components/chart/chart-tooltip.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card/stack-card.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card/stack-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card-empty/stack-card-empty.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card-empty/stack-card-empty.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/snaps/snap-update-alert/snap-update-alert.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-markdown/snap-ui-markdown.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-button/snap-ui-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-settings-page/snap-settings-renderer.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-address/snap-ui-address.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-home-page/snap-home-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-pill/snap-authorship-pill.tsx, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/name/name-details/name-display.tsx, repos/metamask-extension/ui/components/app/name/name-details/shortened-name.tsx, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/name/name-details/formatted-value.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/modals/transaction-confirmed/transaction-confirmed.component.js, repos/metamask-extension/ui/components/app/modals/transaction-confirmed/transaction-confirmed.component.js, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/convert-token-to-nft-modal/convert-token-to-nft-modal.js, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-address/detected-token-address.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/alerts/unconnected-account-alert/unconnected-account-alert.js, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/pages/confirmations/send-utils/send-content/add-recipient/domain-input.component.js, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/ShieldCoverageAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/PendingTransactionAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/NonContractAddressAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/NonContractAddressAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/NonContractAddressAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/AccountTypeMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-list/recipient-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-list/recipient-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/total-row/total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/bridge-time-row/bridge-time-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/bridge-fee-row/bridge-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/bridge-fee-row/bridge-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/required-tokens-row/required-tokens-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/network-statistics/network-statistics.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/network-statistics/network-statistics.js, repos/metamask-extension/ui/pages/confirmations/components/developer/confirmations-developer-options/confirmations-developer-options.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/confirmations-developer-options/confirmations-developer-options.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/wallet-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/dapp-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-agreement.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-gas-limit/advanced-gas-fee-gas-limit.js, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-status-row/transaction-details-status-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-total-row/transaction-details-total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-paid-with-row/transaction-details-paid-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-row/transaction-details-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-bridge-fee-row/transaction-details-bridge-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-hero/transaction-details-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-network-fee-row/transaction-details-network-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-date-row/transaction-details-date-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-date-row/transaction-details-date-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-account-row/transaction-details-account-row.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-change/percentage-change.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-and-amount-change/percentage-and-amount-change.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-and-amount-change/percentage-and-amount-change.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/value-double.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/value-double.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/text.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/date.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/address.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/sort-control/sort-control.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/asset-title.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/snaps/snaps-section/snap-insight.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/snaps/snaps-section/snap-insight.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-footer-coverage-indicator.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/siwe-sign/siwe-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/selected-gas-fee-token/selected-gas-fee-token.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/network-row/network-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/decoded-simulation/decoded-simulation.tsx</t>
-  </si>
-  <si>
-    <t>Tag</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/notifications/NewFeatureTag.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.component.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/useGlobalMenuSections.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/nested-transaction-tag/nested-transaction-tag.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/account-type-label/account-type-label.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-title.tsx</t>
-  </si>
-  <si>
-    <t>SuccessPill</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/transaction-breakdown/transaction-breakdown.component.js, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx</t>
-  </si>
-  <si>
-    <t>Skeleton</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsPointsBalance.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-loading.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-section-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-start-trade-cta-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-start-trade-cta-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance/account-group-balance.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/loading-skeleton.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/loading-skeleton.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/loading-skeleton.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-secondary-display.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-primary-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/token-amount-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/alert-row/alert-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx</t>
-  </si>
-  <si>
-    <t>SensitiveText</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/components/ui/currency-display/currency-display.component.js, repos/metamask-extension/ui/components/ui/currency-display/currency-display.component.js, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance/account-group-balance.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-secondary-display.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-primary-display.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-grouped-symbol-cell.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-protocol-cell.tsx</t>
-  </si>
-  <si>
-    <t>SelectButton</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/selected-asset-button.tsx</t>
-  </si>
-  <si>
-    <t>PopoverHeader</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx</t>
-  </si>
-  <si>
-    <t>Popover</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-filter-menu/index.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/index.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/network-picker.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx</t>
-  </si>
-  <si>
-    <t>PickerNetwork</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/components/multichain/app-header/app-header-locked-content.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx</t>
-  </si>
-  <si>
-    <t>ModalOverlay</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
-  </si>
-  <si>
-    <t>ModalHeader</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-tabs.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
-  </si>
-  <si>
-    <t>ModalFooter</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
-  </si>
-  <si>
-    <t>ModalFocus</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js</t>
-  </si>
-  <si>
-    <t>ModalContent</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
-  </si>
-  <si>
-    <t>ModalBody</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-tabs.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WatchLiquidationStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ReadyToTradeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ChooseLeverageStep.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/CloseAnytimeStep.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
-  </si>
-  <si>
-    <t>Modal</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
-  </si>
-  <si>
-    <t>LottieAnimation</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx</t>
-  </si>
-  <si>
-    <t>Label</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-dropdown/snap-ui-dropdown.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-date-time-picker/snap-ui-date-time-picker.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/index.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/confirm-decrypt-message/confirm-decrypt-message.component.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/pages/swaps/selected-token/selected-token.js, repos/metamask-extension/ui/pages/swaps/notification-page/notification-page.js, repos/metamask-extension/ui/pages/swaps/exchange-rate-display/exchange-rate-display.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/settings/settings-search/settings-search.js, repos/metamask-extension/ui/pages/settings/settings-search/settings-search.js, repos/metamask-extension/ui/pages/settings/settings-search-list/settings-search-list.js, repos/metamask-extension/ui/pages/settings/settings-search-list/settings-search-list.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-list-tab.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/step-progress-bar-item.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/asset/components/asset-breadcrumb.js, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/sender-to-recipient/sender-to-recipient.component.js, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/icon-button/icon-button.stories.tsx, repos/metamask-extension/ui/components/ui/icon-button/icon-button.stories.tsx, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/dropdown/dropdown.js, repos/metamask-extension/ui/components/ui/disclosure/disclosure.js, repos/metamask-extension/ui/components/ui/disclosure/disclosure.js, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu-items/multichain-account-menu-items.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.js, repos/metamask-extension/ui/components/app/selected-account/selected-account.component.js, repos/metamask-extension/ui/components/app/rewards/RewardsErrorToast.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsBadge.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/home-notification/home-notification.component.js, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.stories.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail/transaction-detail.stories.js, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/app/transaction-activity-log/transaction-activity-log-icon/transaction-activity-log-icon.component.js, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-markdown/snap-ui-markdown.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-icon/snap-ui-icon.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-footer-button/snap-ui-footer-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-button/snap-ui-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/name/name-details/name-display.tsx, repos/metamask-extension/ui/components/app/modals/transaction-confirmed/transaction-confirmed.component.js, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/alerts/unconnected-account-alert/unconnected-account-alert.js, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-status-icon/transaction-status-icon.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/selected-gas-fee-token/selected-gas-fee-token.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx</t>
-  </si>
-  <si>
-    <t>HelpText</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-dropdown/snap-ui-dropdown.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-date-time-picker/snap-ui-date-time-picker.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx</t>
-  </si>
-  <si>
-    <t>HeaderBase</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/notification-details/notification-details-header/notification-details-header.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.tsx</t>
-  </si>
-  <si>
-    <t>FormTextField</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/components/ui/form-combo-field/form-combo-field.tsx, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain/import-account/private-key.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-account/json.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-price-input/gas-price-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-input/gas-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-input/snap-ui-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-input/snap-ui-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx</t>
-  </si>
-  <si>
-    <t>FileUploader</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx</t>
-  </si>
-  <si>
-    <t>Container</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/bridge/layout/column.tsx, repos/metamask-extension/ui/pages/bridge/layout/row.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.stories.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.stories.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/create-new-vault/create-new-vault.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-defaults/advanced-gas-fee-defaults.js</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-explorer-links.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-explorer-links.tsx, repos/metamask-extension/ui/components/ui/export-text-container/export-text-container.component.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-account/bottom-buttons.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-section.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-section.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-accounts-page/multichain-edit-accounts-page.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-list-tab.component.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-account/bottom-buttons.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.stories.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/fee-card/fee-card.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-private-key-list-page/multichain-account-private-key-list-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-tx-declined-message.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-button.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/json.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-overview.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permissions-connect-footer/permissions-connect-footer.component.js, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-markdown/snap-ui-markdown.js, repos/metamask-extension/ui/components/app/snaps/update-snap-permission-list/update-snap-permission-list.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-address/detected-token-address.js, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/ShieldCoverageAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/PendingTransactionAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/AccountTypeMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-agreement.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WatchLiquidationStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ChooseLeverageStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/CloseAnytimeStep.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/nft-default-image.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications/notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/confirm-decrypt-message/confirm-decrypt-message.component.js, repos/metamask-extension/ui/pages/bridge/index.tsx, repos/metamask-extension/ui/pages/bridge/index.tsx, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-view.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/redirect-url-icon.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-header/notification-details-header.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-options.js, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/nickname-popover/nickname-popover.component.js, repos/metamask-extension/ui/components/ui/form-combo-field/form-combo-field.tsx, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/callout/callout.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-srp-row/account-show-srp-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-unlocked-content.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/contract-token-values/contract-token-values.js, repos/metamask-extension/ui/pages/confirmations/components/contract-token-values/contract-token-values.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-accounts-page/multichain-edit-accounts-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card/stack-card.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/new-account-modal/new-account-modal.component.js, repos/metamask-extension/ui/components/app/modals/edit-approval-permission/edit-approval-permission.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-options/connected-accounts-list-options.component.js, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/send-utils/send-content/add-recipient/domain-input.component.js, repos/metamask-extension/ui/pages/confirmations/send-utils/send-content/add-recipient/domain-input.component.js, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/scroll-to-bottom/scroll-to-bottom.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/wallet-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/advanced-details-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/block-explorer-link/block-explorer-link.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/index.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/text.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/copy-icon.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-secondary-display.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.stories.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/components/ui/icon-button/icon-button.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-copy-button/notification-detail-copy-button.tsx, repos/metamask-extension/ui/components/multichain/network-filter-menu/index.tsx, repos/metamask-extension/ui/components/multichain/address-copy-button/address-copy-button.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/import-control/import-control.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-read-all-button.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/connected-sites/connected-sites.component.js, repos/metamask-extension/ui/pages/connected-sites/connected-sites.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/confirm-add-suggested-token/confirm-add-suggested-token.js, repos/metamask-extension/ui/pages/swaps/select-quote-popover/select-quote-popover.js, repos/metamask-extension/ui/pages/swaps/select-quote-popover/select-quote-popover.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.stories.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.stories.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.stories.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/account-list.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/account-list.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-button.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures-cancel-button.tsx, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-button/notification-detail-button.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.stories.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.stories.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/home-notification/home-notification.component.js, repos/metamask-extension/ui/components/app/home-notification/home-notification.component.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.stories.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/create-new-vault/create-new-vault.js, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.stories.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.stories.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-icon/edit-gas-fee-icon.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/components/ui/page-container/page-container-footer/page-container-footer.component.js, repos/metamask-extension/ui/components/ui/page-container/page-container-footer/page-container-footer.component.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.stories.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.stories.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-footer-button/snap-ui-footer-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.stories.tsx, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/modals/new-account-modal/new-account-modal.component.js, repos/metamask-extension/ui/components/app/modals/new-account-modal/new-account-modal.component.js, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.stories.tsx, repos/metamask-extension/ui/components/app/modals/hide-token-confirmation-modal/hide-token-confirmation-modal.js, repos/metamask-extension/ui/components/app/modals/hide-token-confirmation-modal/hide-token-confirmation-modal.js, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/flask/experimental-area/experimental-area.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-selection-popover/detected-token-selection-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-selection-popover/detected-token-selection-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/alerts/invalid-custom-network-alert/invalid-custom-network-alert.js, repos/metamask-extension/ui/components/app/alerts/invalid-custom-network-alert/invalid-custom-network-alert.js, repos/metamask-extension/ui/components/app/alerts/unconnected-account-alert/unconnected-account-alert.js, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-footer/confirmation-footer.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-footer/confirmation-footer.js, repos/metamask-extension/ui/pages/confirmations/components/send/amount-recipient/amount-recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-save/advanced-gas-fee-save.js, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-gas-limit/advanced-gas-fee-gas-limit.js, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-icon/edit-gas-icon-button.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/snap-account-redirect.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/snap-account-redirect.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/permissions-connect/permissions-connect.stories.js, repos/metamask-extension/ui/pages/permissions-connect/permissions-connect.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-flow.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-flow.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list.tsx, repos/metamask-extension/ui/pages/notifications/notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-read-all-button.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.stories.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.stories.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.stories.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-item.stories.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-item.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-view.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/url-display-box.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-message.tsx, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-animation.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-toggle-row-component.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/create-password/create-password.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-body/notification-details-body.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-footer/notification-details-footer.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-footer/notification-details-footer.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-detail-row.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/confirmation.js, repos/metamask-extension/ui/pages/confirmations/confirmation/confirmation.js, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/pulsing-circle.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/pulsing-circle.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/segment.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/segment.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/segment.stories.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-list.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-description.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/hollow-circle.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-explorer-links.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-activity-item-tx-segments.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-activity-item-tx-segments.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-list.stories.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-list.stories.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/origin-pill/origin-pill.tsx, repos/metamask-extension/ui/components/ui/metafox-logo/metafox-logo.component.js, repos/metamask-extension/ui/components/ui/logo/logo.stories.js, repos/metamask-extension/ui/components/ui/loading-screen/loading-screen.component.js, repos/metamask-extension/ui/components/ui/loading-screen/loading-screen.component.js, repos/metamask-extension/ui/components/ui/loading-screen/loading-screen.component.js, repos/metamask-extension/ui/components/ui/loading-indicator/loading-indicator.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/export-text-container/export-text-container.component.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/currency-display/currency-display.component.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle/smart-contract-account-toggle.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/multichain-site-cell.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu-items/multichain-account-menu-items.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-srp-row/account-show-srp-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-title/notification-detail-title.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-nft/notification-detail-nft.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-nft/notification-detail-nft.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-collection/notification-detail-collection.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-copy-button/notification-detail-copy-button.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-tabs.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-filter-menu/index.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/bottom-buttons.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/carousel/carousel.tsx, repos/metamask-extension/ui/components/multichain/carousel/carousel.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/badge-status/badge-status.tsx, repos/metamask-extension/ui/components/multichain/badge-status/badge-status.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/app-header/multichain-meta-fox-logo.js, repos/metamask-extension/ui/components/multichain/app-header/app-header.js, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.stories.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.stories.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.stories.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-container.tsx, repos/metamask-extension/ui/components/multichain/address-copy-button/address-copy-button.js, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/account-overview/account-overview-unknown.tsx, repos/metamask-extension/ui/components/multichain/account-overview/account-overview-unknown.tsx, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/app/wallet-overview/coin-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list-item-details/transaction-list-item-details.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/smart-transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permissions-connect-permission-list/permissions-connect-permission-list.js, repos/metamask-extension/ui/components/app/permissions-connect-footer/permissions-connect-footer.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container.component.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/name/name.tsx, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/currency-input/currency-input.js, repos/metamask-extension/ui/components/app/currency-input/currency-input.js, repos/metamask-extension/ui/components/app/currency-input/currency-input.js, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/stories/util.js, repos/metamask-extension/ui/pages/confirmations/confirmation/stories/util.js, repos/metamask-extension/ui/pages/confirmations/confirmation/stories/util.js, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-contract-with-logo/smart-contract-with-logo.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/asset-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/asset-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/amount-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/chart-tooltip.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-empty-state.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-loading.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-search/network-list-search.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-search.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/update-snap-permission-list/update-snap-permission-list.js, repos/metamask-extension/ui/components/app/snaps/update-snap-permission-list/update-snap-permission-list.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-renderer/snap-ui-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-renderer/snap-ui-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-form/snap-ui-form.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-dropdown/snap-ui-dropdown.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-settings-page/snap-settings-renderer.tsx, repos/metamask-extension/ui/components/app/snaps/snap-settings-page/snap-settings-renderer.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-address/snap-ui-address.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-home-page/snap-home-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-home-page/snap-home-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-pill/snap-authorship-pill.tsx, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hide-token-confirmation-modal/hide-token-confirmation-modal.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/index.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.stories.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-address/detected-token-address.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-details/detected-token-details.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-details/detected-token-details.js, repos/metamask-extension/ui/components/app/assets/defi-list/defi-list.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance/account-group-balance.tsx, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/components/transactions/nested-transaction-tag/nested-transaction-tag.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-filter-input/recipient-filter-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-filter-input/asset-filter-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount-recipient/amount-recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount-recipient/amount-recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/total-row/total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/total-row/total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/required-tokens-row/required-tokens-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/simulation-settings-modal/simulation-settings-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/dataTree.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/scroll-to-bottom/scroll-to-bottom.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/scroll-to-bottom/scroll-to-bottom.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/wallet-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/dapp-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/dapp-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/advanced-details-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/blockaid-loading-indicator/blockaid-loading-indicator.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-agreement.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-defaults/advanced-gas-fee-defaults.js, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-status-row/transaction-details-status-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-paid-with-row/transaction-details-paid-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-row/transaction-details-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-hero/transaction-details-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-date-row/transaction-details-date-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-change/percentage-change.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-and-amount-change/percentage-and-amount-change.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/index.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/value-double.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/text.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/section.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/date.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/currency.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/address.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/address.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/nft-default-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/sort-control/sort-control.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/sort-control/sort-control.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/snaps/snaps-section/snaps-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/typed-sign-data-v1/typedSignDataV1.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/typed-sign-data-v1/typedSignDataV1.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/typed-sign-data/typedSignData.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/typed-sign-data/typedSignData.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/token-transfer.stories.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/nft-token-transfer/nft-token-transfer.stories.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/native-transfer/native-transfer.stories.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-footer-coverage-indicator.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-footer-coverage-indicator.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/content/content.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/alert-row/alert-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/alert-row/alert-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/revoke-set-approval-for-all-static-simulation/revoke-set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/revoke-set-approval-for-all-static-simulation/revoke-set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/revoke-set-approval-for-all-static-simulation/revoke-set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/revoke-set-approval-for-all-static-simulation/revoke-set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/siwe-sign/siwe-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/static-simulation/static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/transaction-data/transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/transaction-data/transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/transaction-data/transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/transaction-data/transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/selected-gas-fee-token/selected-gas-fee-token.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-icon/gas-fee-token-icon.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-icon/gas-fee-token-icon.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/network-row/network-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-details/gas-fees-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-toast/gas-fee-token-toast.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/batched-approval-function/batched-approval-function.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/confirm-loader/confirm-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/batch/nested-transaction-data/nested-transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/revoke-static-simulation/revoke-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/revoke-static-simulation/revoke-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/revoke-static-simulation/revoke-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/revoke-static-simulation/revoke-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/permit-simulation/permit-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/permit-simulation/permit-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx</t>
-  </si>
-  <si>
-    <t>BannerTip</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx</t>
-  </si>
-  <si>
-    <t>BannerBase</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx</t>
-  </si>
-  <si>
-    <t>BannerAlert</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/confirm-add-suggested-token/confirm-add-suggested-token.js, repos/metamask-extension/ui/pages/confirm-add-suggested-token/confirm-add-suggested-token.js, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-private-key-list-page/multichain-account-private-key-list-page.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/typography/typography.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/menu/menu.stories.js, repos/metamask-extension/ui/components/ui/icon-with-fallback/icon-with-fallback.stories.js, repos/metamask-extension/ui/components/ui/icon-border/icon-border.stories.js, repos/metamask-extension/ui/components/ui/chip/chip.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/detected-token-banner/detected-token-banner.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/contact-list/contact-list.component.js, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-error-banner.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-error-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-error-message/simulation-error-message.js, repos/metamask-extension/ui/pages/confirmations/components/simulation-error-message/simulation-error-message.js, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/components/app/snaps/snap-update-alert/snap-update-alert.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-banner/snap-ui-banner.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-detection-notice-nfts-tab/nfts-detection-notice-nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-detection-notice-import-nfts/nfts-detection-notice-import-nfts.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-collection/notification-detail-collection.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-asset/notification-detail-asset.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/multichain/badge-status/badge-status.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/app/transaction-list-item/smart-transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/token-icon/token-icon.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-details/detected-token-details.js, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/asset-cell-badge.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-collection/notification-detail-collection.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-asset/notification-detail-asset.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-asset/notification-detail-asset.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-asset/notification-detail-asset.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/pages/confirmations/components/token-icon/token-icon.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-details/detected-token-details.js, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/asset-cell-badge.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-icon/gas-fee-token-icon.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/app/transaction-list-item/smart-transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/token-icon/token-icon.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/asset-pill.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-details/detected-token-details.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/asset-cell-badge.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/network-row/network-row.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-info/notification-detail-info.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/app/transaction-icon/transaction-icon.js, repos/metamask-extension/ui/components/app/transaction-icon/transaction-icon.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/components/ui/origin-pill/origin-pill.tsx, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-sites-list.component.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-icon/snap-icon.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-icon/snap-icon.tsx</t>
-  </si>
-  <si>
-    <t>AvatarAccount</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/components/ui/identicon/identicon.component.js, repos/metamask-extension/ui/components/multichain/toast/toast.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/app/preferred-avatar/preferred-avatar.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx</t>
-  </si>
-  <si>
-    <t>AvatarGroup</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/network-picker.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/permission-item.tsx, repos/metamask-extension/ui/components/app/chain-badge/chain-badge.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/selected-asset-button.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/components/app/perps/perps-token-logo/perps-token-logo.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/selected-asset-button.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/native-amount-row.tsx</t>
-  </si>
-  <si>
-    <t>BadgeCount</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx</t>
-  </si>
-  <si>
-    <t>BadgeCountSize</t>
-  </si>
-  <si>
-    <t>BadgeIcon</t>
-  </si>
-  <si>
-    <t>BadgeNetwork</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx</t>
-  </si>
-  <si>
-    <t>BadgeStatus</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx</t>
-  </si>
-  <si>
-    <t>BadgeStatusStatus</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx, repos/metamask-extension/ui/components/app/chain-badge/chain-badge.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/selected-asset-button.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx</t>
-  </si>
-  <si>
-    <t>BadgeWrapperPosition</t>
-  </si>
-  <si>
-    <t>Blockies</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/rewards/index.tsx, repos/metamask-extension/ui/pages/settings/settings-toggle-item.tsx, repos/metamask-extension/ui/pages/settings/settings-toggle-item.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/create-account/create-account.component.js, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/shield-banner-animation.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/shield-banner-animation.tsx, repos/metamask-extension/ui/pages/settings/experimental-tab/experimental-tab.tsx, repos/metamask-extension/ui/pages/settings/backup-and-sync-tab/backup-and-sync-tab.tsx, repos/metamask-extension/ui/pages/settings/backup-and-sync-tab/backup-and-sync-tab.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/setting.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/setting.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/setting.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/metamask-wordmark-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/metamask-wordmark-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/fox-appear-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/fox-appear-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/wallet-ready-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/wallet-ready-animation.tsx, repos/metamask-extension/ui/pages/multichain-accounts/smart-account-page/smart-account-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-private-key-list-page/multichain-account-private-key-list-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-address-list-page/multichain-account-address-list-page.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/components/ui/tabs/tabs.tsx, repos/metamask-extension/ui/components/ui/tabs/tabs.tsx, repos/metamask-extension/ui/components/ui/tabs/tabs.tsx, repos/metamask-extension/ui/components/ui/tab-empty-state/tab-empty-state.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-network-group-with-default-address/multichain-account-network-group-with-default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-aggregated-list-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-aggregated-list-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-aggregated-list-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-network-group/multichain-account-network-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain/menu-items/discover-menu-item.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/useGlobalMenuSections.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/useGlobalMenuSections.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/permission-item.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/permission-item.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-unlocked-content.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-illustration-animation.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-illustration-animation.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorToast.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsBadge.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsBadge.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsBadge.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/balance-empty-state/balance-empty-state.tsx, repos/metamask-extension/ui/components/app/balance-empty-state/balance-empty-state.tsx, repos/metamask-extension/ui/components/app/balance-empty-state/balance-empty-state.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/api-error-handler/api-error-handler.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/crypto-account-display.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row-container.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-price-input/gas-price-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-input/gas-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-date-time-picker/snap-ui-date-time-picker.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/ProgressIndicator.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/ProgressIndicator.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/perps/start-trade-cta/start-trade-cta.tsx, repos/metamask-extension/ui/components/app/perps/start-trade-cta/start-trade-cta.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/ProgressIndicator.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/ProgressIndicator.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialAnimation.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialAnimation.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-section-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-section-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-section-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-start-trade-cta-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-empty-state/perps-empty-state.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/perps-candlestick-chart/perps-candlestick-chart.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/quote-swap-simulation-details/quote-swap-simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/quote-swap-simulation-details/quote-swap-simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/quote-swap-simulation-details/quote-swap-simulation-details.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/token-transfer/token-transfer-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/review-permissions/review-gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WatchLiquidationStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WatchLiquidationStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WatchLiquidationStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ReadyToTradeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ReadyToTradeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ReadyToTradeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ChooseLeverageStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ChooseLeverageStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ChooseLeverageStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/CloseAnytimeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/CloseAnytimeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/CloseAnytimeStep.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-title.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/estimated-changes.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-icon-animation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-icon-animation.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/direction-tabs/direction-tabs.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/token-amount-row.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/native-amount-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/date-and-time-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/quote-transaction-data/quoted-transaction-data.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/components/ui/tab-empty-state/tab-empty-state.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list-item-details/transaction-list-item-details.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/cancel-button/cancel-button.js, repos/metamask-extension/ui/components/app/balance-empty-state/balance-empty-state.tsx, repos/metamask-extension/ui/components/app/api-error-handler/api-error-handler.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/manage-shield-plan/manage-shield-plan.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/reactivate-button.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WatchLiquidationStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ReadyToTradeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ChooseLeverageStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/CloseAnytimeStep.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/start-trade-cta/start-trade-cta.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/direction-tabs/direction-tabs.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/direction-tabs/direction-tabs.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx</t>
-  </si>
-  <si>
-    <t>ButtonBaseSize</t>
-  </si>
-  <si>
-    <t>ButtonHero</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/multichain-accounts/smart-account-page/smart-account-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-private-key-list-page/multichain-account-private-key-list-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-address-list-page/multichain-account-address-list-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/add-wallet-page/add-wallet-page.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/token-transfer/token-transfer-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/review-permissions/review-gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-network-group-with-default-address/multichain-account-network-group-with-default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-aggregated-list-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-unlocked-content.tsx, repos/metamask-extension/ui/components/app/rewards/AddRewardsAccount.tsx, repos/metamask-extension/ui/components/app/rewards/AddRewardsAccount.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/musd/claim-bonus-badge.tsx, repos/metamask-extension/ui/components/app/api-error-handler/api-error-handler.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/crypto-account-display.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/perps/start-trade-cta/start-trade-cta.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-empty-state/perps-empty-state.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx</t>
-  </si>
-  <si>
-    <t>IconName</t>
-  </si>
-  <si>
-    <t>Jazzicon</t>
-  </si>
-  <si>
-    <t>Maskicon</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-plan.tsx, repos/metamask-extension/ui/pages/settings/settings-toggle-item.tsx, repos/metamask-extension/ui/pages/settings/settings-toggle-item.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/payment-method-row.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/migrate-to-split-state-test.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/perps/market-list/index.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/setting.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/core/defi-referral-consent/defi-referral-consent.tsx, repos/metamask-extension/ui/pages/multichain-accounts/add-wallet-page/add-wallet-page.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/components/ui/tab-empty-state/tab-empty-state.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx, repos/metamask-extension/ui/components/ui/menu/menu-item.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-network-group-with-default-address/multichain-account-network-group-with-default-address.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-aggregated-list-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-aggregated-list-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/global-menu-drawer.stories.tsx, repos/metamask-extension/ui/components/multichain/global-menu/global-menu-list.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/permission-item.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/permission-item.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/non-evm-activity-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list.tsx, repos/metamask-extension/ui/components/multichain/activity-v2/activity-list.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsBadge.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsErrorBanner.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-view.tsx, repos/metamask-extension/ui/components/app/musd/claim-bonus-badge.tsx, repos/metamask-extension/ui/components/app/musd/claim-bonus-badge.tsx, repos/metamask-extension/ui/components/app/balance-empty-state/balance-empty-state.tsx, repos/metamask-extension/ui/components/app/balance-empty-state/balance-empty-state.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/api-error-handler/api-error-handler.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-list/claims-list.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/crypto-account-display.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/external/add-ethereum-chain/add-ethereum-chain.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-price-input/gas-price-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-estimate-list-item/gas-estimate-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/components/ui/tabs/tab/tab.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/perps/start-trade-cta/start-trade-cta.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/position-card/position-card.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/transaction-card/transaction-card.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-tab-control-bar/perps-tab-control-bar.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-slider/perps-slider.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-market-balance-actions/perps-market-balance-actions.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-recent-activity/perps-recent-activity.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/order-card/order-card.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row/market-row.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/dropdown/dropdown.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/quote-swap-simulation-details/quote-swap-simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/dapp-swap-comparison-banner/dapp-swap-comparison-banner.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/lazy-asset-list.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/review-permissions/review-gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-group-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permissions-cell-connection-list-item.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WhatArePerpsStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WatchLiquidationStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/WatchLiquidationStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/GoLongShortStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ReadyToTradeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ReadyToTradeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ChooseLeverageStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/ChooseLeverageStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/CloseAnytimeStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/steps/CloseAnytimeStep.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/direction-tabs/direction-tabs.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/direction-tabs/direction-tabs.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/order-summary/order-summary.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/close-amount-section/close-amount-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/native-token-periodic-details.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/native-amount-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/erc20-token-periodic-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/date-and-time-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/date-and-time-row.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/design-system/design-system.stories.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/default-address.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/app/rewards/AddRewardsAccount.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx</t>
-  </si>
-  <si>
-    <t>TextVariant</t>
-  </si>
-  <si>
-    <t>Path</t>
-  </si>
-  <si>
     <t>ui/components/component-library/text-field/text-field.tsx</t>
   </si>
   <si>
     <t>ui/components/component-library/tag/tag.tsx</t>
   </si>
   <si>
+    <t>ui/components/component-library/sensitive-text/sensitive-text.tsx</t>
+  </si>
+  <si>
     <t>ui/components/component-library/success-pill/success-pill.tsx</t>
   </si>
   <si>
     <t>ui/components/component-library/skeleton/skeleton.tsx</t>
   </si>
   <si>
-    <t>ui/components/component-library/sensitive-text/sensitive-text.tsx</t>
-  </si>
-  <si>
     <t>ui/components/component-library/select-button/select-button.tsx</t>
   </si>
   <si>
     <t>ui/components/component-library/popover-header/popover-header.tsx</t>
   </si>
   <si>
+    <t>ui/components/component-library/picker-network/picker-network.tsx</t>
+  </si>
+  <si>
+    <t>ui/components/component-library/modal-overlay/modal-overlay.tsx</t>
+  </si>
+  <si>
     <t>ui/components/component-library/popover/popover.tsx</t>
   </si>
   <si>
-    <t>ui/components/component-library/picker-network/picker-network.tsx</t>
-  </si>
-  <si>
-    <t>ui/components/component-library/modal-overlay/modal-overlay.tsx</t>
+    <t>ui/components/component-library/modal-focus/modal-focus.tsx</t>
   </si>
   <si>
     <t>ui/components/component-library/modal-footer/modal-footer.tsx</t>
-  </si>
-  <si>
-    <t>ui/components/component-library/modal-focus/modal-focus.tsx</t>
   </si>
   <si>
     <t>ui/components/component-library/modal-body/modal-body.tsx</t>
@@ -1009,10 +979,10 @@
         <v>6</v>
       </c>
       <c r="D2">
-        <v>1276</v>
+        <v>1272</v>
       </c>
       <c r="E2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -1049,10 +1019,10 @@
         <v>12</v>
       </c>
       <c r="D4">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E4">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F4" t="s">
         <v>14</v>
@@ -1109,7 +1079,7 @@
         <v>20</v>
       </c>
       <c r="D7">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E7" t="s">
         <v>21</v>
@@ -1149,10 +1119,10 @@
         <v>20</v>
       </c>
       <c r="D9">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E9">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="F9" t="s">
         <v>27</v>
@@ -1169,10 +1139,10 @@
         <v>30</v>
       </c>
       <c r="D10">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E10">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F10" t="s">
         <v>31</v>
@@ -1189,7 +1159,7 @@
         <v>32</v>
       </c>
       <c r="D11">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E11">
         <v>20</v>
@@ -1212,7 +1182,7 @@
         <v>15</v>
       </c>
       <c r="E12">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F12" t="s">
         <v>37</v>
@@ -1229,10 +1199,10 @@
         <v>38</v>
       </c>
       <c r="D13">
-        <v>1593</v>
+        <v>1591</v>
       </c>
       <c r="E13">
-        <v>696</v>
+        <v>708</v>
       </c>
       <c r="F13" t="s">
         <v>40</v>
@@ -1269,7 +1239,7 @@
         <v>44</v>
       </c>
       <c r="D15">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="E15">
         <v>10</v>
@@ -1289,7 +1259,7 @@
         <v>47</v>
       </c>
       <c r="D16">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="E16">
         <v>10</v>
@@ -1369,10 +1339,10 @@
         <v>26</v>
       </c>
       <c r="D20">
-        <v>3852</v>
+        <v>3838</v>
       </c>
       <c r="E20">
-        <v>1418</v>
+        <v>1434</v>
       </c>
       <c r="F20" t="s">
         <v>59</v>
@@ -1411,7 +1381,7 @@
         <v>65</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
         <v>66</v>
@@ -1425,7 +1395,7 @@
         <v>65</v>
       </c>
       <c r="C3">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D3" t="s">
         <v>68</v>
@@ -1439,7 +1409,7 @@
         <v>65</v>
       </c>
       <c r="C4">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
         <v>70</v>
@@ -1453,7 +1423,7 @@
         <v>65</v>
       </c>
       <c r="C5">
-        <v>1276</v>
+        <v>1272</v>
       </c>
       <c r="D5" t="s">
         <v>71</v>
@@ -1467,7 +1437,7 @@
         <v>65</v>
       </c>
       <c r="C6">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
         <v>73</v>
@@ -1481,7 +1451,7 @@
         <v>65</v>
       </c>
       <c r="C7">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
         <v>75</v>
@@ -1495,7 +1465,7 @@
         <v>65</v>
       </c>
       <c r="C8">
-        <v>117</v>
+        <v>5</v>
       </c>
       <c r="D8" t="s">
         <v>77</v>
@@ -1509,7 +1479,7 @@
         <v>65</v>
       </c>
       <c r="C9">
-        <v>24</v>
+        <v>117</v>
       </c>
       <c r="D9" t="s">
         <v>79</v>
@@ -1551,7 +1521,7 @@
         <v>65</v>
       </c>
       <c r="C12">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D12" t="s">
         <v>85</v>
@@ -1565,7 +1535,7 @@
         <v>65</v>
       </c>
       <c r="C13">
-        <v>3</v>
+        <v>105</v>
       </c>
       <c r="D13" t="s">
         <v>87</v>
@@ -1579,7 +1549,7 @@
         <v>65</v>
       </c>
       <c r="C14">
-        <v>106</v>
+        <v>20</v>
       </c>
       <c r="D14" t="s">
         <v>89</v>
@@ -1593,7 +1563,7 @@
         <v>65</v>
       </c>
       <c r="C15">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D15" t="s">
         <v>91</v>
@@ -1607,7 +1577,7 @@
         <v>65</v>
       </c>
       <c r="C16">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="D16" t="s">
         <v>93</v>
@@ -1621,7 +1591,7 @@
         <v>65</v>
       </c>
       <c r="C17">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="D17" t="s">
         <v>95</v>
@@ -1635,7 +1605,7 @@
         <v>65</v>
       </c>
       <c r="C18">
-        <v>111</v>
+        <v>42</v>
       </c>
       <c r="D18" t="s">
         <v>97</v>
@@ -1649,7 +1619,7 @@
         <v>65</v>
       </c>
       <c r="C19">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D19" t="s">
         <v>99</v>
@@ -1663,7 +1633,7 @@
         <v>65</v>
       </c>
       <c r="C20">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D20" t="s">
         <v>101</v>
@@ -1685,27 +1655,27 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22" t="s">
         <v>104</v>
-      </c>
-      <c r="B22" t="s">
-        <v>65</v>
-      </c>
-      <c r="C22">
-        <v>18</v>
-      </c>
-      <c r="D22" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>9</v>
+        <v>105</v>
       </c>
       <c r="B23" t="s">
         <v>65</v>
       </c>
       <c r="C23">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D23" t="s">
         <v>106</v>
@@ -1713,27 +1683,27 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>107</v>
       </c>
       <c r="B24" t="s">
         <v>65</v>
       </c>
       <c r="C24">
-        <v>216</v>
+        <v>18</v>
       </c>
       <c r="D24" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>108</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
         <v>65</v>
       </c>
       <c r="C25">
-        <v>18</v>
+        <v>215</v>
       </c>
       <c r="D25" t="s">
         <v>109</v>
@@ -1747,7 +1717,7 @@
         <v>65</v>
       </c>
       <c r="C26">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="D26" t="s">
         <v>111</v>
@@ -1761,7 +1731,7 @@
         <v>65</v>
       </c>
       <c r="C27">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="D27" t="s">
         <v>113</v>
@@ -1789,7 +1759,7 @@
         <v>65</v>
       </c>
       <c r="C29">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D29" t="s">
         <v>117</v>
@@ -1825,13 +1795,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B32" t="s">
         <v>65</v>
       </c>
       <c r="C32">
-        <v>42</v>
+        <v>103</v>
       </c>
       <c r="D32" t="s">
         <v>120</v>
@@ -1839,13 +1809,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
         <v>65</v>
       </c>
       <c r="C33">
-        <v>108</v>
+        <v>156</v>
       </c>
       <c r="D33" t="s">
         <v>121</v>
@@ -1853,13 +1823,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="B34" t="s">
         <v>65</v>
       </c>
       <c r="C34">
-        <v>157</v>
+        <v>41</v>
       </c>
       <c r="D34" t="s">
         <v>122</v>
@@ -1895,27 +1865,27 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>125</v>
       </c>
       <c r="B37" t="s">
         <v>65</v>
       </c>
       <c r="C37">
-        <v>1593</v>
+        <v>2</v>
       </c>
       <c r="D37" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>126</v>
+        <v>38</v>
       </c>
       <c r="B38" t="s">
         <v>65</v>
       </c>
       <c r="C38">
-        <v>2</v>
+        <v>1591</v>
       </c>
       <c r="D38" t="s">
         <v>127</v>
@@ -1971,7 +1941,7 @@
         <v>65</v>
       </c>
       <c r="C42">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="D42" t="s">
         <v>133</v>
@@ -1985,7 +1955,7 @@
         <v>65</v>
       </c>
       <c r="C43">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="D43" t="s">
         <v>134</v>
@@ -2041,7 +2011,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2112,7 +2082,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B7">
         <v>10</v>
@@ -2123,7 +2093,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B8">
         <v>10</v>
@@ -2159,18 +2129,18 @@
         <v>148</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>149</v>
+        <v>41</v>
       </c>
       <c r="B12">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
         <v>150</v>
@@ -2178,40 +2148,40 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13">
+        <v>708</v>
+      </c>
+      <c r="C13" t="s">
         <v>151</v>
-      </c>
-      <c r="B13">
-        <v>2</v>
-      </c>
-      <c r="C13" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>153</v>
+        <v>20</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="C14" t="s">
-        <v>26</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B15">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -2222,188 +2192,78 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>156</v>
+        <v>32</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C17" t="s">
-        <v>26</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="B18">
-        <v>696</v>
+        <v>2</v>
       </c>
       <c r="C18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B19">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C19" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="B20">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="C20" t="s">
-        <v>159</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>160</v>
+        <v>6</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>455</v>
       </c>
       <c r="C21" t="s">
-        <v>26</v>
+        <v>158</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>161</v>
+        <v>30</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="C22" t="s">
-        <v>26</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="B23">
-        <v>20</v>
+        <v>1450</v>
       </c>
       <c r="C23" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B24">
-        <v>2</v>
-      </c>
-      <c r="C24" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>12</v>
-      </c>
-      <c r="B25">
-        <v>82</v>
-      </c>
-      <c r="C25" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>165</v>
-      </c>
-      <c r="B26">
-        <v>0</v>
-      </c>
-      <c r="C26" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>9</v>
-      </c>
-      <c r="B27">
-        <v>0</v>
-      </c>
-      <c r="C27" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>166</v>
-      </c>
-      <c r="B28">
-        <v>0</v>
-      </c>
-      <c r="C28" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>167</v>
-      </c>
-      <c r="B29">
-        <v>0</v>
-      </c>
-      <c r="C29" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>6</v>
-      </c>
-      <c r="B30">
-        <v>456</v>
-      </c>
-      <c r="C30" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>30</v>
-      </c>
-      <c r="B31">
-        <v>15</v>
-      </c>
-      <c r="C31" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>170</v>
-      </c>
-      <c r="B32">
-        <v>0</v>
-      </c>
-      <c r="C32" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>58</v>
-      </c>
-      <c r="B33">
-        <v>1436</v>
-      </c>
-      <c r="C33" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2423,7 +2283,7 @@
         <v>60</v>
       </c>
       <c r="B1" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="C1" t="s">
         <v>62</v>
@@ -2434,16 +2294,16 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>161</v>
       </c>
       <c r="C2">
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -2451,10 +2311,10 @@
         <v>69</v>
       </c>
       <c r="B3" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C3">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
         <v>70</v>
@@ -2465,10 +2325,10 @@
         <v>72</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="C4">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
         <v>73</v>
@@ -2479,10 +2339,10 @@
         <v>74</v>
       </c>
       <c r="B5" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="C5">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="D5" t="s">
         <v>75</v>
@@ -2493,10 +2353,10 @@
         <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="C6">
-        <v>117</v>
+        <v>5</v>
       </c>
       <c r="D6" t="s">
         <v>77</v>
@@ -2507,10 +2367,10 @@
         <v>78</v>
       </c>
       <c r="B7" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="C7">
-        <v>24</v>
+        <v>117</v>
       </c>
       <c r="D7" t="s">
         <v>79</v>
@@ -2521,7 +2381,7 @@
         <v>80</v>
       </c>
       <c r="B8" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -2535,7 +2395,7 @@
         <v>82</v>
       </c>
       <c r="B9" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -2549,10 +2409,10 @@
         <v>84</v>
       </c>
       <c r="B10" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="C10">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D10" t="s">
         <v>85</v>
@@ -2563,10 +2423,10 @@
         <v>86</v>
       </c>
       <c r="B11" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="C11">
-        <v>3</v>
+        <v>105</v>
       </c>
       <c r="D11" t="s">
         <v>87</v>
@@ -2577,10 +2437,10 @@
         <v>88</v>
       </c>
       <c r="B12" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="C12">
-        <v>106</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s">
         <v>89</v>
@@ -2591,10 +2451,10 @@
         <v>92</v>
       </c>
       <c r="B13" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="C13">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="D13" t="s">
         <v>93</v>
@@ -2602,16 +2462,16 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B14" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="C14">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -2619,10 +2479,10 @@
         <v>98</v>
       </c>
       <c r="B15" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="C15">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D15" t="s">
         <v>99</v>
@@ -2633,10 +2493,10 @@
         <v>100</v>
       </c>
       <c r="B16" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="C16">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D16" t="s">
         <v>101</v>
@@ -2647,7 +2507,7 @@
         <v>102</v>
       </c>
       <c r="B17" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="C17">
         <v>2</v>
@@ -2658,44 +2518,44 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B18" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="C18">
         <v>18</v>
       </c>
       <c r="D18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B19" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="C19">
         <v>18</v>
       </c>
       <c r="D19" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B20" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="C20">
         <v>2</v>
       </c>
       <c r="D20" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -2703,7 +2563,7 @@
         <v>114</v>
       </c>
       <c r="B21" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -2717,10 +2577,10 @@
         <v>116</v>
       </c>
       <c r="B22" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="C22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D22" t="s">
         <v>117</v>
@@ -2728,16 +2588,16 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B23" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="C23">
         <v>2</v>
       </c>
       <c r="D23" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -2745,7 +2605,7 @@
         <v>128</v>
       </c>
       <c r="B24" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="C24">
         <v>2</v>
@@ -2759,7 +2619,7 @@
         <v>130</v>
       </c>
       <c r="B25" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="C25">
         <v>64</v>
@@ -2776,7 +2636,7 @@
         <v>26</v>
       </c>
       <c r="C26">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="D26" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
fix: use anti-fragile component name matching instead of suffix filtering
- Match exported names to folder/file names (architectural pattern)
- Removed fragile suffix-based filtering (was excluding BadgeStatus)
- Now correctly includes: BadgeStatus, Blockies, Jazzicon, Maskicon
- Also includes temp-components: ButtonAnimated, TextOrChildren
- Updated counts: Extension 21→25, Mobile 29→35 components
- Regenerate 2026-02-27 metrics with accurate component counts
</commit_message>
<xml_diff>
--- a/metrics/extension-component-metrics-2026-02-27.xlsx
+++ b/metrics/extension-component-metrics-2026-02-27.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="189">
   <si>
     <t>Deprecated Component</t>
   </si>
@@ -70,24 +70,24 @@
     <t>5.56%</t>
   </si>
   <si>
+    <t>ButtonPrimary</t>
+  </si>
+  <si>
+    <t>ui/components/component-library/button-primary/button-primary.tsx</t>
+  </si>
+  <si>
+    <t>Button</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>ButtonSecondary</t>
   </si>
   <si>
     <t>ui/components/component-library/button-secondary/button-secondary.tsx</t>
   </si>
   <si>
-    <t>Button</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>ButtonPrimary</t>
-  </si>
-  <si>
-    <t>ui/components/component-library/button-primary/button-primary.tsx</t>
-  </si>
-  <si>
     <t>ui/components/component-library/button/button.tsx</t>
   </si>
   <si>
@@ -148,6 +148,33 @@
     <t>31.58%</t>
   </si>
   <si>
+    <t>AvatarToken</t>
+  </si>
+  <si>
+    <t>ui/components/component-library/avatar-token/avatar-token.tsx</t>
+  </si>
+  <si>
+    <t>27.03%</t>
+  </si>
+  <si>
+    <t>AvatarIcon</t>
+  </si>
+  <si>
+    <t>ui/components/component-library/avatar-icon/avatar-icon.tsx</t>
+  </si>
+  <si>
+    <t>12.50%</t>
+  </si>
+  <si>
+    <t>AvatarFavicon</t>
+  </si>
+  <si>
+    <t>ui/components/component-library/avatar-favicon/avatar-favicon.tsx</t>
+  </si>
+  <si>
+    <t>6.25%</t>
+  </si>
+  <si>
     <t>AvatarNetwork</t>
   </si>
   <si>
@@ -157,33 +184,6 @@
     <t>14.29%</t>
   </si>
   <si>
-    <t>AvatarToken</t>
-  </si>
-  <si>
-    <t>ui/components/component-library/avatar-token/avatar-token.tsx</t>
-  </si>
-  <si>
-    <t>27.03%</t>
-  </si>
-  <si>
-    <t>AvatarIcon</t>
-  </si>
-  <si>
-    <t>ui/components/component-library/avatar-icon/avatar-icon.tsx</t>
-  </si>
-  <si>
-    <t>12.50%</t>
-  </si>
-  <si>
-    <t>AvatarFavicon</t>
-  </si>
-  <si>
-    <t>ui/components/component-library/avatar-favicon/avatar-favicon.tsx</t>
-  </si>
-  <si>
-    <t>6.25%</t>
-  </si>
-  <si>
     <t>AvatarBase</t>
   </si>
   <si>
@@ -208,28 +208,28 @@
     <t>File Paths</t>
   </si>
   <si>
+    <t>Textarea</t>
+  </si>
+  <si>
+    <t>ui/components/component-library/textarea/textarea.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/components/ui/textarea/textarea.stories.js, repos/metamask-extension/ui/components/ui/textarea/textarea.stories.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx</t>
+  </si>
+  <si>
     <t>TextFieldSearch</t>
   </si>
   <si>
-    <t>ui/components/component-library/text-field-search/deprecated/text-field-search.js</t>
-  </si>
-  <si>
     <t>repos/metamask-extension/ui/pages/swaps/list-with-search/list-with-search.js, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-search/network-list-search.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-search.tsx, repos/metamask-extension/ui/components/app/import-token/token-search/token-search.component.js, repos/metamask-extension/ui/pages/perps/market-list/components/search-input/search-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-filter-input/recipient-filter-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-filter-input/asset-filter-input.tsx</t>
   </si>
   <si>
-    <t>Textarea</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/components/ui/textarea/textarea.stories.js, repos/metamask-extension/ui/components/ui/textarea/textarea.stories.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx</t>
+    <t>repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/formatted-counter.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/confirm-add-suggested-token/confirm-add-suggested-token.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/loading-swaps-quotes/loading-swaps-quotes.js, repos/metamask-extension/ui/pages/swaps/loading-swaps-quotes/loading-swaps-quotes.js, repos/metamask-extension/ui/pages/swaps/notification-page/notification-page.js, repos/metamask-extension/ui/pages/swaps/notification-page/notification-page.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/swaps/list-with-search/list-with-search.js, repos/metamask-extension/ui/pages/swaps/fee-card/fee-card.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/url-display-box.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-message.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-detail-row.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-activity-item-tx-segments.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-description.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-description.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-tx-declined-message.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-no-fee-message.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-info-text.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-button.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle/smart-contract-account-toggle.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu-items/multichain-account-menu-items.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-srp-row/account-show-srp-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/token-balance/token-balance.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/origin-pill/origin-pill.tsx, repos/metamask-extension/ui/components/ui/numeric-input/numeric-input.component.js, repos/metamask-extension/ui/components/ui/metafox-logo/metafox-logo.stories.js, repos/metamask-extension/ui/components/ui/logo/logo.stories.js, repos/metamask-extension/ui/components/ui/icon-button/icon-button.tsx, repos/metamask-extension/ui/components/ui/icon-button/icon-button.tsx, repos/metamask-extension/ui/components/ui/icon/icon.stories.js, repos/metamask-extension/ui/components/ui/icon/icon.stories.js, repos/metamask-extension/ui/components/ui/icon/icon.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/export-text-container/export-text-container.component.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/disclosure/disclosure.js, repos/metamask-extension/ui/components/ui/delineator/delineator.stories.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.stories.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.stories.tsx, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/confusable/confusable.component.js, repos/metamask-extension/ui/components/ui/confusable/confusable.component.js, repos/metamask-extension/ui/components/ui/chip/chip.js, repos/metamask-extension/ui/components/ui/callout/callout.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/actionable-message/actionable-message.stories.js, repos/metamask-extension/ui/components/ui/actionable-message/actionable-message.stories.js, repos/metamask-extension/ui/components/ui/actionable-message/actionable-message.stories.js, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-text/notification-list-item-text.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-text/notification-list-item-text.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-title/notification-detail-title.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-title/notification-detail-title.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-collection/notification-detail-collection.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-info/notification-detail-info.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-info/notification-detail-info.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-asset/notification-detail-asset.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-address/notification-detail-address.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/menu-items/view-explorer-menu-item.tsx, repos/metamask-extension/ui/components/multichain/menu-items/account-details-menu-item.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/json.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/app-header/app-header-unlocked-content.tsx, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/selected-account/selected-account.component.js, repos/metamask-extension/ui/components/app/selected-account/selected-account.component.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permissions-connect-footer/permissions-connect-footer.component.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.stories.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.stories.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/name/name.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/snap-account-success-message/SnapAccountSuccessMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/snap-account-error-message/SnapAccountErrorMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-contract-with-logo/smart-contract-with-logo.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/amount-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/asset-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/contract-token-values/contract-token-values.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/pages/asset/components/chart/chart-tooltip.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card-empty/stack-card-empty.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card-empty/stack-card-empty.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card/stack-card.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card/stack-card.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/snaps/snap-update-alert/snap-update-alert.js, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-markdown/snap-ui-markdown.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-button/snap-ui-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address/snap-ui-address.tsx, repos/metamask-extension/ui/components/app/snaps/snap-settings-page/snap-settings-renderer.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-home-page/snap-home-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-pill/snap-authorship-pill.tsx, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/name/name-details/name-display.tsx, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/name/name-details/formatted-value.tsx, repos/metamask-extension/ui/components/app/name/name-details/shortened-name.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-confirmed/transaction-confirmed.component.js, repos/metamask-extension/ui/components/app/modals/transaction-confirmed/transaction-confirmed.component.js, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/convert-token-to-nft-modal/convert-token-to-nft-modal.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-address/detected-token-address.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/alerts/unconnected-account-alert/unconnected-account-alert.js, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/send-utils/send-content/add-recipient/domain-input.component.js, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/ShieldCoverageAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/NonContractAddressAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/NonContractAddressAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/NonContractAddressAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/PendingTransactionAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/AccountTypeMessage.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-list/recipient-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-list/recipient-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/total-row/total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/bridge-time-row/bridge-time-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/bridge-fee-row/bridge-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/bridge-fee-row/bridge-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/required-tokens-row/required-tokens-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/network-statistics/network-statistics.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/network-statistics/network-statistics.js, repos/metamask-extension/ui/pages/confirmations/components/developer/confirmations-developer-options/confirmations-developer-options.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/confirmations-developer-options/confirmations-developer-options.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/wallet-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/dapp-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-agreement.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-gas-limit/advanced-gas-fee-gas-limit.js, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-total-row/transaction-details-total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-row/transaction-details-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-status-row/transaction-details-status-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-paid-with-row/transaction-details-paid-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-date-row/transaction-details-date-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-date-row/transaction-details-date-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-account-row/transaction-details-account-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-network-fee-row/transaction-details-network-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-hero/transaction-details-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-bridge-fee-row/transaction-details-bridge-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-change/percentage-change.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-and-amount-change/percentage-and-amount-change.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-and-amount-change/percentage-and-amount-change.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/value-double.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/value-double.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/date.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/address.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/text.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/sort-control/sort-control.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/asset-title.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/snaps/snaps-section/snap-insight.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/snaps/snaps-section/snap-insight.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-footer-coverage-indicator.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/selected-gas-fee-token/selected-gas-fee-token.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/network-row/network-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/siwe-sign/siwe-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/decoded-simulation/decoded-simulation.tsx</t>
   </si>
   <si>
     <t>TextField</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/formatted-counter.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/confirm-add-suggested-token/confirm-add-suggested-token.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/smart-transaction-status/smart-transaction-status.js, repos/metamask-extension/ui/pages/swaps/notification-page/notification-page.js, repos/metamask-extension/ui/pages/swaps/notification-page/notification-page.js, repos/metamask-extension/ui/pages/swaps/list-with-search/list-with-search.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/swaps/loading-swaps-quotes/loading-swaps-quotes.js, repos/metamask-extension/ui/pages/swaps/loading-swaps-quotes/loading-swaps-quotes.js, repos/metamask-extension/ui/pages/swaps/fee-card/fee-card.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/url-display-box.tsx, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/swaps/awaiting-signatures/awaiting-signatures.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-message.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-detail-row.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-description.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-description.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-activity-item-tx-segments.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-tx-declined-message.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-no-fee-message.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-info-text.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-button.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle/smart-contract-account-toggle.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu-items/multichain-account-menu-items.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-srp-row/account-show-srp-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/token-balance/token-balance.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/slider/slider.component.js, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/origin-pill/origin-pill.tsx, repos/metamask-extension/ui/components/ui/numeric-input/numeric-input.component.js, repos/metamask-extension/ui/components/ui/metafox-logo/metafox-logo.stories.js, repos/metamask-extension/ui/components/ui/logo/logo.stories.js, repos/metamask-extension/ui/components/ui/icon-button/icon-button.tsx, repos/metamask-extension/ui/components/ui/icon-button/icon-button.tsx, repos/metamask-extension/ui/components/ui/icon/icon.stories.js, repos/metamask-extension/ui/components/ui/icon/icon.stories.js, repos/metamask-extension/ui/components/ui/icon/icon.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/export-text-container/export-text-container.component.js, repos/metamask-extension/ui/components/ui/delineator/delineator.stories.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.stories.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.stories.tsx, repos/metamask-extension/ui/components/ui/disclosure/disclosure.js, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/confusable/confusable.component.js, repos/metamask-extension/ui/components/ui/confusable/confusable.component.js, repos/metamask-extension/ui/components/ui/chip/chip.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.js, repos/metamask-extension/ui/components/ui/actionable-message/actionable-message.stories.js, repos/metamask-extension/ui/components/ui/actionable-message/actionable-message.stories.js, repos/metamask-extension/ui/components/ui/actionable-message/actionable-message.stories.js, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/box/box.stories.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-text/notification-list-item-text.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-text/notification-list-item-text.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-title/notification-detail-title.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-title/notification-detail-title.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-info/notification-detail-info.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-info/notification-detail-info.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-collection/notification-detail-collection.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-address/notification-detail-address.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-asset/notification-detail-asset.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.stories.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/menu-items/view-explorer-menu-item.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/menu-items/account-details-menu-item.js, repos/metamask-extension/ui/components/multichain/import-account/json.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-unlocked-content.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/srp-input/srp-input.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/selected-account/selected-account.component.js, repos/metamask-extension/ui/components/app/selected-account/selected-account.component.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.stories.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.stories.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/permissions-connect-footer/permissions-connect-footer.component.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-account-balance-header/network-account-balance-header.js, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/name/name.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-result/snap-result.js, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.component.js, repos/metamask-extension/ui/pages/confirmations/components/snap-account-success-message/SnapAccountSuccessMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/snap-account-error-message/SnapAccountErrorMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-contract-with-logo/smart-contract-with-logo.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/fiat-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/asset-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/amount-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/confirmations/components/contract-token-values/contract-token-values.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/asset/components/chart/chart-tooltip.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card-empty/stack-card-empty.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card-empty/stack-card-empty.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card/stack-card.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card/stack-card.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-update-alert/snap-update-alert.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-markdown/snap-ui-markdown.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-button/snap-ui-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address/snap-ui-address.tsx, repos/metamask-extension/ui/components/app/snaps/snap-settings-page/snap-settings-renderer.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-permission-cell/snap-permission-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-page/snap-home-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-pill/snap-authorship-pill.tsx, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/name/name-details/shortened-name.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-display.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/formatted-value.tsx, repos/metamask-extension/ui/components/app/modals/transaction-confirmed/transaction-confirmed.component.js, repos/metamask-extension/ui/components/app/modals/transaction-confirmed/transaction-confirmed.component.js, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/convert-token-to-nft-modal/convert-token-to-nft-modal.js, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-address/detected-token-address.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/alerts/unconnected-account-alert/unconnected-account-alert.js, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/send-utils/send-content/add-recipient/domain-input.component.js, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/ShieldCoverageAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/NonContractAddressAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/NonContractAddressAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/NonContractAddressAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/PendingTransactionAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/AccountTypeMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-list/recipient-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-list/recipient-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/total-row/total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/required-tokens-row/required-tokens-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/bridge-fee-row/bridge-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/bridge-fee-row/bridge-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/bridge-time-row/bridge-time-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/network-statistics/network-statistics.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/network-statistics/network-statistics.js, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-tooltip/edit-gas-tooltip.js, repos/metamask-extension/ui/pages/confirmations/components/developer/confirmations-developer-options/confirmations-developer-options.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/confirmations-developer-options/confirmations-developer-options.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/wallet-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/dapp-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-agreement.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-gas-limit/advanced-gas-fee-gas-limit.js, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-row/transaction-details-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-status-row/transaction-details-status-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-total-row/transaction-details-total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-network-fee-row/transaction-details-network-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-paid-with-row/transaction-details-paid-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-date-row/transaction-details-date-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-date-row/transaction-details-date-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-account-row/transaction-details-account-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-bridge-fee-row/transaction-details-bridge-fee-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-hero/transaction-details-hero.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-change/percentage-change.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-and-amount-change/percentage-and-amount-change.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-and-amount-change/percentage-and-amount-change.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/value-double.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/value-double.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/text.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/date.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/address.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/sort-control/sort-control.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/asset-title.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/snaps/snaps-section/snap-insight.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/snaps/snaps-section/snap-insight.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/subscription-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-footer-coverage-indicator.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/network-row/network-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/selected-gas-fee-token/selected-gas-fee-token.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/siwe-sign/siwe-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/decoded-simulation/decoded-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx</t>
+    <t>repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/ui/text-field/text-field.stories.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/perps/edit-margin/edit-margin-expandable.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/limit-price-input/limit-price-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/leverage-slider/leverage-slider.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/amount-input/amount-input.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/components/auto-close-section/auto-close-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
   </si>
   <si>
     <t>Tag</t>
@@ -238,22 +238,22 @@
     <t>repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/notifications/NewFeatureTag.tsx, repos/metamask-extension/ui/pages/settings/info-tab/info-tab.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/global-menu-drawer/useGlobalMenuSections.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/components/app/perps/order-entry/order-entry.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/nested-transaction-tag/nested-transaction-tag.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/account-type-label/account-type-label.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/asset.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-title.tsx</t>
   </si>
   <si>
+    <t>Skeleton</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsPointsBalance.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-loading.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-section-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-start-trade-cta-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-start-trade-cta-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance/account-group-balance.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/loading-skeleton.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/loading-skeleton.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/loading-skeleton.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-secondary-display.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-primary-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/alert-row/alert-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/token-amount-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx</t>
+  </si>
+  <si>
+    <t>SuccessPill</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/transaction-breakdown/transaction-breakdown.component.js, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx</t>
+  </si>
+  <si>
     <t>SensitiveText</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.tsx, repos/metamask-extension/ui/components/ui/currency-display/currency-display.component.js, repos/metamask-extension/ui/components/ui/currency-display/currency-display.component.js, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance/account-group-balance.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-secondary-display.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-protocol-cell.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-grouped-symbol-cell.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-primary-display.tsx</t>
-  </si>
-  <si>
-    <t>SuccessPill</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/transaction-breakdown/transaction-breakdown.component.js, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx</t>
-  </si>
-  <si>
-    <t>Skeleton</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-home-page.tsx, repos/metamask-extension/ui/pages/perps/perps-market-detail-page.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/transaction-shield.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsPointsBalance.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/membership-header.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/button-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-loading.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-start-trade-cta-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-start-trade-cta-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-home-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-card-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-control-bar-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-section-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-detail-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-activity-page-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/perps/perps-skeletons/perps-balance-actions-skeleton.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance/account-group-balance.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/perps/market-list/components/market-row-skeleton/market-row-skeleton.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/musd-claim-info/musd-claim-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/info.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/loading-skeleton.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/loading-skeleton.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/loading-skeleton.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/review-gator-permission-item.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-secondary-display.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-primary-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shield-subscription-approve/shield-subscription-approve-loader.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/alert-row/alert-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-permission/token-amount-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx</t>
+    <t>repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.tsx, repos/metamask-extension/ui/components/ui/currency-display/currency-display.component.js, repos/metamask-extension/ui/components/ui/currency-display/currency-display.component.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance/account-group-balance.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-secondary-display.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-primary-display.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-protocol-cell.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-grouped-symbol-cell.tsx</t>
   </si>
   <si>
     <t>SelectButton</t>
@@ -277,19 +277,31 @@
     <t>ModalOverlay</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
   </si>
   <si>
     <t>Popover</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-filter-menu/index.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/index.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/network-picker.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx</t>
+    <t>repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-hovered-list/multichain-hovered-address-rows-hovered-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-filter-menu/index.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/perps/perps-candle-period-selector/perps-candle-period-selector.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/index.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/network-picker.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx</t>
   </si>
   <si>
     <t>ModalHeader</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/network-manager/network-tabs.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-tabs.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+  </si>
+  <si>
+    <t>ModalFooter</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+  </si>
+  <si>
+    <t>ModalContent</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
   </si>
   <si>
     <t>ModalFocus</t>
@@ -298,28 +310,25 @@
     <t>repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/account-list-item-menu/account-list-item-menu.js</t>
   </si>
   <si>
-    <t>ModalContent</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
-  </si>
-  <si>
-    <t>ModalFooter</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
-  </si>
-  <si>
     <t>ModalBody</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-tabs.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+    <t>repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-tabs.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/rewards/RewardsQRCode.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep2.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep4.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep1.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingStep3.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingIntroStep.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
   </si>
   <si>
     <t>Modal</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-payment-modal.tsx, repos/metamask-extension/ui/pages/shield-plan/shield-rewards-modal.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/bridge/token-insights-modal/token-insights-modal.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/address-qr-code-modal/address-qr-code-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-wallet-modal/add-wallet-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-manager.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-permissions-modal/disconnect-permissions-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/shield-entry-modal/shield-entry-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/cancel-speedup-popover/cancel-speedup-popover.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/network-selector/network-selector.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/components/cancel-membership-modal.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/account-selector/account-selector.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-popover/edit-gas-fee-popover.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/rewards/onboarding/OnboardingModal.tsx, repos/metamask-extension/ui/components/app/perps/perps-tutorial-modal/PerpsTutorialModal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/transaction-already-confirmed/transaction-already-confirmed.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/pna25-modal/pna25-modal.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/add-funds-modal/add-funds-modal.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-gas-price-modal/advanced-gas-price-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/pay-with-modal/pay-with-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/advanced-eip1559-modal/advanced-eip1559-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/modals/estimates-modal/estimates-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-modal/transaction-details-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/bridge-asset-picker/index.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/edit-spending-cap-modal/edit-spending-cap-modal.tsx</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-dropdown/snap-ui-dropdown.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-date-time-picker/snap-ui-date-time-picker.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/index.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx</t>
   </si>
   <si>
     <t>LottieAnimation</t>
@@ -328,28 +337,19 @@
     <t>repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-animation.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx</t>
-  </si>
-  <si>
-    <t>Label</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-date-time-picker/snap-ui-date-time-picker.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-dropdown/snap-ui-dropdown.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/index.tsx</t>
+    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/confirm-decrypt-message/confirm-decrypt-message.component.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/pages/swaps/selected-token/selected-token.js, repos/metamask-extension/ui/pages/swaps/notification-page/notification-page.js, repos/metamask-extension/ui/pages/swaps/exchange-rate-display/exchange-rate-display.js, repos/metamask-extension/ui/pages/settings/settings-search-list/settings-search-list.js, repos/metamask-extension/ui/pages/settings/settings-search-list/settings-search-list.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/settings/settings-search/settings-search.js, repos/metamask-extension/ui/pages/settings/settings-search/settings-search.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-list-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/step-progress-bar-item.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/asset-breadcrumb.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu-items/multichain-account-menu-items.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/ui/sender-to-recipient/sender-to-recipient.component.js, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/icon-button/icon-button.stories.tsx, repos/metamask-extension/ui/components/ui/icon-button/icon-button.stories.tsx, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/dropdown/dropdown.js, repos/metamask-extension/ui/components/ui/disclosure/disclosure.js, repos/metamask-extension/ui/components/ui/disclosure/disclosure.js, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.js, repos/metamask-extension/ui/components/app/selected-account/selected-account.component.js, repos/metamask-extension/ui/components/app/rewards/RewardsErrorToast.tsx, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/home-notification/home-notification.component.js, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.stories.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail/transaction-detail.stories.js, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/transaction-activity-log/transaction-activity-log-icon/transaction-activity-log-icon.component.js, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-markdown/snap-ui-markdown.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-icon/snap-ui-icon.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-footer-button/snap-ui-footer-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-button/snap-ui-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/name/name-details/name-display.tsx, repos/metamask-extension/ui/components/app/modals/transaction-confirmed/transaction-confirmed.component.js, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/alerts/unconnected-account-alert/unconnected-account-alert.js, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-status-icon/transaction-status-icon.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/selected-gas-fee-token/selected-gas-fee-token.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx</t>
   </si>
   <si>
     <t>HelpText</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-date-time-picker/snap-ui-date-time-picker.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-dropdown/snap-ui-dropdown.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/confirm-decrypt-message/confirm-decrypt-message.component.js, repos/metamask-extension/ui/helpers/utils/permission.js, repos/metamask-extension/ui/pages/swaps/notification-page/notification-page.js, repos/metamask-extension/ui/pages/swaps/selected-token/selected-token.js, repos/metamask-extension/ui/pages/swaps/exchange-rate-display/exchange-rate-display.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/settings/settings-search-list/settings-search-list.js, repos/metamask-extension/ui/pages/settings/settings-search-list/settings-search-list.js, repos/metamask-extension/ui/pages/settings/settings-search/settings-search.js, repos/metamask-extension/ui/pages/settings/settings-search/settings-search.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-list-tab.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/asset-breadcrumb.js, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/step-progress-bar-item.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu-items/multichain-account-menu-items.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/tooltip/tooltip.stories.js, repos/metamask-extension/ui/components/ui/sender-to-recipient/sender-to-recipient.component.js, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/icon-button/icon-button.stories.tsx, repos/metamask-extension/ui/components/ui/icon-button/icon-button.stories.tsx, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/form-field/form-field.stories.js, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/dropdown/dropdown.js, repos/metamask-extension/ui/components/ui/disclosure/disclosure.js, repos/metamask-extension/ui/components/ui/disclosure/disclosure.js, repos/metamask-extension/ui/components/ui/definition-list/definition-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/toast-master/toast-master.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.stories.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.js, repos/metamask-extension/ui/components/app/selected-account/selected-account.component.js, repos/metamask-extension/ui/components/app/rewards/RewardsErrorToast.tsx, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/home-notification/home-notification.component.js, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail-item/transaction-detail-item.stories.js, repos/metamask-extension/ui/pages/confirmations/components/transaction-detail/transaction-detail.stories.js, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-button/edit-gas-fee-button.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/app/transaction-activity-log/transaction-activity-log-icon/transaction-activity-log-icon.component.js, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.tsx, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-markdown/snap-ui-markdown.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-icon/snap-ui-icon.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-footer-button/snap-ui-footer-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-button/snap-ui-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/name/name-details/name-display.tsx, repos/metamask-extension/ui/components/app/modals/transaction-confirmed/transaction-confirmed.component.js, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/alerts/unconnected-account-alert/unconnected-account-alert.js, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-status-icon/transaction-status-icon.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/selected-gas-fee-token/selected-gas-fee-token.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx</t>
+    <t>repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-dropdown/snap-ui-dropdown.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-date-time-picker/snap-ui-date-time-picker.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx</t>
   </si>
   <si>
     <t>FormTextField</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/ui/form-combo-field/form-combo-field.tsx, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/private-key.js, repos/metamask-extension/ui/components/multichain/import-account/json.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-price-input/gas-price-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-input/gas-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-input/snap-ui-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-input/snap-ui-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx</t>
+    <t>repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/ui/form-combo-field/form-combo-field.tsx, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/json.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/import-account/private-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/transaction-shield-tab/claims-form/claims-form.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/confirmations/components/priority-fee-input/priority-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/max-base-fee-input/max-base-fee-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-price-input/gas-price-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-input/gas-input.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-input/snap-ui-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-input/snap-ui-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx</t>
   </si>
   <si>
     <t>HeaderBase</t>
@@ -370,25 +370,28 @@
     <t>repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/basic-functionality-required/basic-functionality-required.tsx, repos/metamask-extension/ui/pages/bridge/layout/row.tsx, repos/metamask-extension/ui/pages/bridge/layout/column.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.stories.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.stories.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/create-new-vault/create-new-vault.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-defaults/advanced-gas-fee-defaults.js</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-explorer-links.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-explorer-links.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/ui/export-text-container/export-text-container.component.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/bottom-buttons.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-section.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-accounts-page/multichain-edit-accounts-page.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/fee-card/fee-card.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-private-key-list-page/multichain-account-private-key-list-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-tx-declined-message.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-button.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/import-account/json.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-overview.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permissions-connect-footer/permissions-connect-footer.component.js, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/update-snap-permission-list/update-snap-permission-list.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-markdown/snap-ui-markdown.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-address/detected-token-address.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/ShieldCoverageAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/PendingTransactionAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/AccountTypeMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-agreement.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/nft-default-image.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications/notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/confirm-decrypt-message/confirm-decrypt-message.component.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/bridge/index.tsx, repos/metamask-extension/ui/pages/bridge/index.tsx, repos/metamask-extension/ui/pages/snaps/snap-view/snap-view.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/redirect-url-icon.tsx, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-header/notification-details-header.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-options.js, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-srp-row/account-show-srp-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/nickname-popover/nickname-popover.component.js, repos/metamask-extension/ui/components/ui/form-combo-field/form-combo-field.tsx, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/callout/callout.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-unlocked-content.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/contract-token-values/contract-token-values.js, repos/metamask-extension/ui/pages/confirmations/components/contract-token-values/contract-token-values.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-accounts-page/multichain-edit-accounts-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card/stack-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/new-account-modal/new-account-modal.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/edit-approval-permission/edit-approval-permission.component.js, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-options/connected-accounts-list-options.component.js, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/send-utils/send-content/add-recipient/domain-input.component.js, repos/metamask-extension/ui/pages/confirmations/send-utils/send-content/add-recipient/domain-input.component.js, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/scroll-to-bottom/scroll-to-bottom.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/wallet-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/advanced-details-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/block-explorer-link/block-explorer-link.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/index.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/text.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/copy-icon.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.stories.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-secondary-display.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx</t>
-  </si>
-  <si>
-    <t>repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-list-tab.component.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/bottom-buttons.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.stories.tsx</t>
+    <t>repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.stories.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.stories.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/create-new-vault/create-new-vault.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-defaults/advanced-gas-fee-defaults.js</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/swaps/transaction-settings/transaction-settings.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-list-tab.component.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/bottom-buttons.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.stories.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-explorer-links.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-explorer-links.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/ui/export-text-container/export-text-container.component.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/bottom-buttons.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-section.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-accounts-page/multichain-edit-accounts-page.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/token-cell.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/swaps-banner-alert/swaps-banner-alert.js, repos/metamask-extension/ui/pages/swaps/fee-card/fee-card.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-private-key-list-page/multichain-account-private-key-list-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/quotes/bridge-quotes-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-tx-declined-message.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-input-group.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-button.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/import-account/json.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-overview.tsx, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permissions-connect-footer/permissions-connect-footer.component.js, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/network-connection-banner/network-connection-banner.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list.component.js, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/app/snaps/update-snap-permission-list/update-snap-permission-list.js, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-markdown/snap-ui-markdown.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-link/snap-ui-link.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-address/detected-token-address.js, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/ShieldCoverageAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/PendingTransactionAlertMessage.tsx, repos/metamask-extension/ui/pages/confirmations/hooks/alerts/transactions/AccountTypeMessage.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-agreement.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/nft-default-image.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/perps/perps-activity-page.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications/notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/confirm-decrypt-message/confirm-decrypt-message.component.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/bridge/index.tsx, repos/metamask-extension/ui/pages/bridge/index.tsx, repos/metamask-extension/ui/pages/snaps/snap-view/snap-view.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/redirect-url-icon.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-header/notification-details-header.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/bridge/quotes/multichain-bridge-quote-card.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-options.js, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-srp-row/account-show-srp-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-private-key-row/account-show-private-key-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.stories.tsx, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/popover/popover.component.js, repos/metamask-extension/ui/components/ui/nickname-popover/nickname-popover.component.js, repos/metamask-extension/ui/components/ui/form-combo-field/form-combo-field.tsx, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/callout/callout.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-unlocked-content.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-options.js, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/contract-token-values/contract-token-values.js, repos/metamask-extension/ui/pages/confirmations/components/contract-token-values/contract-token-values.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-accounts-page/multichain-edit-accounts-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/carousel/stack-card/stack-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/new-account-modal/new-account-modal.component.js, repos/metamask-extension/ui/components/app/modals/edit-approval-permission/edit-approval-permission.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-options/connected-accounts-list-options.component.js, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/send-utils/send-content/add-recipient/domain-input.component.js, repos/metamask-extension/ui/pages/confirmations/send-utils/send-content/add-recipient/domain-input.component.js, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/scroll-to-bottom/scroll-to-bottom.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/wallet-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/advanced-details-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/block-explorer-link/block-explorer-link.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/index.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/copy-icon.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/text.tsx, repos/metamask-extension/ui/components/app/assets/token-cell/cells/token-cell-secondary-display.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.stories.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/header/header.stories.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx</t>
   </si>
   <si>
     <t>repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/components/ui/icon-button/icon-button.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-copy-button/notification-detail-copy-button.tsx, repos/metamask-extension/ui/components/multichain/network-filter-menu/index.tsx, repos/metamask-extension/ui/components/multichain/address-copy-button/address-copy-button.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-display/edit-gas-display.component.js, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/import-control/import-control.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-read-all-button.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/connected-sites/connected-sites.component.js, repos/metamask-extension/ui/pages/connected-sites/connected-sites.component.js, repos/metamask-extension/ui/pages/confirm-add-suggested-token/confirm-add-suggested-token.js, repos/metamask-extension/ui/pages/swaps/select-quote-popover/select-quote-popover.js, repos/metamask-extension/ui/pages/swaps/select-quote-popover/select-quote-popover.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.stories.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.stories.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.stories.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/account-list.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/account-list.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures-cancel-button.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-button.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.stories.tsx, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/multichain/notification-detail-button/notification-detail-button.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.stories.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.stories.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/home-notification/home-notification.component.js, repos/metamask-extension/ui/components/app/home-notification/home-notification.component.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.stories.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/create-new-vault/create-new-vault.js, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.stories.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.stories.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-icon/edit-gas-fee-icon.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/ui/page-container/page-container-footer/page-container-footer.component.js, repos/metamask-extension/ui/components/ui/page-container/page-container-footer/page-container-footer.component.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.stories.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.stories.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-footer-button/snap-ui-footer-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/new-account-modal/new-account-modal.component.js, repos/metamask-extension/ui/components/app/modals/new-account-modal/new-account-modal.component.js, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.stories.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hide-token-confirmation-modal/hide-token-confirmation-modal.js, repos/metamask-extension/ui/components/app/modals/hide-token-confirmation-modal/hide-token-confirmation-modal.js, repos/metamask-extension/ui/components/app/flask/experimental-area/experimental-area.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-selection-popover/detected-token-selection-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-selection-popover/detected-token-selection-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/alerts/unconnected-account-alert/unconnected-account-alert.js, repos/metamask-extension/ui/components/app/alerts/invalid-custom-network-alert/invalid-custom-network-alert.js, repos/metamask-extension/ui/components/app/alerts/invalid-custom-network-alert/invalid-custom-network-alert.js, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-footer/confirmation-footer.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-footer/confirmation-footer.js, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount-recipient/amount-recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-save/advanced-gas-fee-save.js, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-gas-limit/advanced-gas-fee-gas-limit.js, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-icon/edit-gas-icon-button.tsx</t>
+    <t>repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-read-all-button.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/keychains/reveal-seed.js, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/connected-sites/connected-sites.component.js, repos/metamask-extension/ui/pages/connected-sites/connected-sites.component.js, repos/metamask-extension/ui/pages/confirm-add-suggested-token/confirm-add-suggested-token.js, repos/metamask-extension/ui/pages/swaps/select-quote-popover/select-quote-popover.js, repos/metamask-extension/ui/pages/swaps/select-quote-popover/select-quote-popover.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.stories.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.stories.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.stories.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/index.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/account-list.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/account-list.js, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-cta-button.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures-cancel-button.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.stories.tsx, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/ui/button/button.stories.js, repos/metamask-extension/ui/components/multichain/notification-detail-button/notification-detail-button.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-sites-modal.tsx, repos/metamask-extension/ui/components/multichain/disconnect-all-modal/disconnect-all-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.stories.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.stories.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/home-notification/home-notification.component.js, repos/metamask-extension/ui/components/app/home-notification/home-notification.component.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.stories.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/create-new-vault/create-new-vault.js, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.stories.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.stories.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/set-approval-for-all-warning/set-approval-for-all-warning.js, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-popover/edit-gas-popover.component.js, repos/metamask-extension/ui/pages/confirmations/components/edit-gas-fee-icon/edit-gas-fee-icon.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/components/ui/page-container/page-container-footer/page-container-footer.component.js, repos/metamask-extension/ui/components/ui/page-container/page-container-footer/page-container-footer.component.js, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.stories.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/SRPQuiz/SRPQuiz.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-footer-button/snap-ui-footer-button.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.stories.tsx, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/new-account-modal/new-account-modal.component.js, repos/metamask-extension/ui/components/app/modals/new-account-modal/new-account-modal.component.js, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.stories.tsx, repos/metamask-extension/ui/components/app/modals/hide-token-confirmation-modal/hide-token-confirmation-modal.js, repos/metamask-extension/ui/components/app/modals/hide-token-confirmation-modal/hide-token-confirmation-modal.js, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/flask/experimental-area/experimental-area.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-selection-popover/detected-token-selection-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-selection-popover/detected-token-selection-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/alerts/unconnected-account-alert/unconnected-account-alert.js, repos/metamask-extension/ui/components/app/alerts/invalid-custom-network-alert/invalid-custom-network-alert.js, repos/metamask-extension/ui/components/app/alerts/invalid-custom-network-alert/invalid-custom-network-alert.js, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-footer/confirmation-footer.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-footer/confirmation-footer.js, repos/metamask-extension/ui/pages/confirmations/components/send/amount-recipient/amount-recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/ledger-info/ledger-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-save/advanced-gas-fee-save.js, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-gas-limit/advanced-gas-fee-gas-limit.js, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-icon/edit-gas-icon-button.tsx</t>
+  </si>
+  <si>
+    <t>repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/snap-account-redirect.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/snap-account-redirect.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/permissions-connect/permissions-connect.stories.js, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-flow.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-flow.tsx, repos/metamask-extension/ui/pages/permissions-connect/permissions-connect.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-read-all-button.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-item.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-item.stories.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.stories.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.stories.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.stories.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-view.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/url-display-box.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-animation.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-message.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-toggle-row-component.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/create-password/create-password.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-footer/notification-details-footer.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-footer/notification-details-footer.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-body/notification-details-body.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/confirmation.js, repos/metamask-extension/ui/pages/confirmations/confirmation/confirmation.js, repos/metamask-extension/ui/pages/bridge/transaction-details/segment.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/segment.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/hollow-circle.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-detail-row.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/pulsing-circle.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/pulsing-circle.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/segment.stories.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-explorer-links.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-activity-item-tx-segments.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-activity-item-tx-segments.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-list.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-list.stories.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-list.stories.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-description.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle/smart-contract-account-toggle.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/multichain-site-cell.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu-items/multichain-account-menu-items.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-srp-row/account-show-srp-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/origin-pill/origin-pill.tsx, repos/metamask-extension/ui/components/ui/metafox-logo/metafox-logo.component.js, repos/metamask-extension/ui/components/ui/logo/logo.stories.js, repos/metamask-extension/ui/components/ui/loading-indicator/loading-indicator.js, repos/metamask-extension/ui/components/ui/loading-screen/loading-screen.component.js, repos/metamask-extension/ui/components/ui/loading-screen/loading-screen.component.js, repos/metamask-extension/ui/components/ui/loading-screen/loading-screen.component.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/export-text-container/export-text-container.component.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/currency-display/currency-display.component.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-nft/notification-detail-nft.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-nft/notification-detail-nft.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-title/notification-detail-title.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-collection/notification-detail-collection.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-copy-button/notification-detail-copy-button.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-tabs.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-filter-menu/index.tsx, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/bottom-buttons.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/carousel/carousel.tsx, repos/metamask-extension/ui/components/multichain/carousel/carousel.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/badge-status/badge-status.tsx, repos/metamask-extension/ui/components/multichain/badge-status/badge-status.tsx, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.stories.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.stories.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.stories.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header-container.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header.js, repos/metamask-extension/ui/components/multichain/app-header/multichain-meta-fox-logo.js, repos/metamask-extension/ui/components/multichain/address-copy-button/address-copy-button.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/account-overview/account-overview-unknown.tsx, repos/metamask-extension/ui/components/multichain/account-overview/account-overview-unknown.tsx, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/app/wallet-overview/coin-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list-item-details/transaction-list-item-details.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/smart-transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permissions-connect-permission-list/permissions-connect-permission-list.js, repos/metamask-extension/ui/components/app/permissions-connect-footer/permissions-connect-footer.component.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container.component.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/name/name.tsx, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/currency-input/currency-input.js, repos/metamask-extension/ui/components/app/currency-input/currency-input.js, repos/metamask-extension/ui/components/app/currency-input/currency-input.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/stories/util.js, repos/metamask-extension/ui/pages/confirmations/confirmation/stories/util.js, repos/metamask-extension/ui/pages/confirmations/confirmation/stories/util.js, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-contract-with-logo/smart-contract-with-logo.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/amount-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/asset-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/asset-pill.tsx, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/percentage-buttons/percentage-buttons.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/pay-token-amount/pay-token-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/gas-timing/gas-timing.component.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/gas-details-item/gas-details-item.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/fee-details-component/fee-details-component.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/confirmations/components/confirmation-warning-modal/confirmation-warning-modal.js, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart.tsx, repos/metamask-extension/ui/pages/bridge/prepare/components/destination-account-list-item.tsx, repos/metamask-extension/ui/pages/asset/components/chart/chart-tooltip.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-price.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-loading.tsx, repos/metamask-extension/ui/pages/asset/components/chart/asset-chart-empty-state.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/multichain-edit-networks-page/multichain-edit-networks-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/tool-tip/multichain-site-cell-tooltip.tsx, repos/metamask-extension/ui/components/multichain-accounts/permissions/permission-review-page/multichain-review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/avatar-group/multichain-avatar-group.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/review-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/permissions-page.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/permissions-page/connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/gator-permissions-page.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.tsx, repos/metamask-extension/ui/components/multichain/pages/page/page.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/select-rpc-url-modal/select-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-search/network-list-search.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-rpc-url-modal/add-rpc-url-modal.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-type-selection/wallet-details-account-type-selection.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/popular-network-list/popular-network-list.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-card.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-block-explorer-modal/add-block-explorer-modal.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/add-non-evm-account/add-non-evm-account.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multichain-accounts/wallet-details-account-item/wallet-details-account-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/srp-list/srp-list-item.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/solana-account-creation-prompt.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-search.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/multi-srp/select-srp/select-srp.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/asset-picker-modal-network.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/multichain/asset-picker-amount/asset-picker-modal/AssetList.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/srp-quiz-modal/QuizContent/QuizContent.tsx, repos/metamask-extension/ui/components/app/snaps/update-snap-permission-list/update-snap-permission-list.js, repos/metamask-extension/ui/components/app/snaps/update-snap-permission-list/update-snap-permission-list.js, repos/metamask-extension/ui/components/app/snaps/snap-version/snap-external-pill.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-selector/snap-ui-selector.stories.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-renderer/snap-ui-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-renderer/snap-ui-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-radio-group/snap-ui-radio-group.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-form/snap-ui-form.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-dropdown/snap-ui-dropdown.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-checkbox/snap-ui-checkbox.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-card/snap-ui-card.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-file-input/snap-ui-file-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-asset-selector/snap-ui-asset-selector.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address/snap-ui-address.tsx, repos/metamask-extension/ui/components/app/snaps/snap-settings-page/snap-settings-renderer.tsx, repos/metamask-extension/ui/components/app/snaps/snap-settings-page/snap-settings-renderer.tsx, repos/metamask-extension/ui/components/app/snaps/snap-remove-warning/snap-remove-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-ui-address-input/snap-ui-address-input.tsx, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-privacy-warning/snap-privacy-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-permissions-list/snap-permissions-list.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-metadata-modal/snap-metadata-modal.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-link-warning/snap-link-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-list-item/snap-list-item.js, repos/metamask-extension/ui/components/app/snaps/snap-home-page/snap-home-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-home-page/snap-home-renderer.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-home-menu/snap-home-menu.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-delineator/snap-delineator.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-connect-cell/snap-connect-cell.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-pill/snap-authorship-pill.tsx, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/snap-install-warning/snap-install-warning.js, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/snaps/show-more/show-more.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-header/snap-authorship-header.js, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-account-list-item.tsx, repos/metamask-extension/ui/components/app/snaps/keyring-snap-removal-warning/keyring-snap-removal-warning.tsx, repos/metamask-extension/ui/components/app/snaps/install-error/install-error.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/copyable/copyable.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/snaps/snap-authorship-expanded/snap-authorship-expanded.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/qr-hardware-popover/qr-hardware-sign-request/player.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container-content/permission-page-container-content.component.js, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/app/modals/visit-support-data-consent-modal/visit-support-data-consent-modal.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/modals/turn-on-metamask-notifications/turn-on-metamask-notifications.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/name/name-details/name-details.tsx, repos/metamask-extension/ui/components/app/modals/keyring-snap-removal-modal/keyring-snap-removal-result-modal.tsx, repos/metamask-extension/ui/components/app/modals/hold-to-reveal-modal/hold-to-reveal-modal.tsx, repos/metamask-extension/ui/components/app/modals/hide-token-confirmation-modal/hide-token-confirmation-modal.js, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/hardware-wallet-error-modal/hardware-wallet-error-modal.tsx, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/modals/customize-nonce/customize-nonce.component.js, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-toggle/backup-and-sync-toggle.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/identity/backup-and-sync-features-toggles/backup-and-sync-features-toggles.tsx, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/token-list/token-list.component.js, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-selector-custom-import/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/index.tsx, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-values/detected-token-values.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-details/detected-token-details.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-details/detected-token-details.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.stories.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-aggregators/detected-token-aggregators.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-ignored-popover/detected-token-ignored-popover.js, repos/metamask-extension/ui/components/app/detected-token/detected-token-address/detected-token-address.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/connected-accounts-list/connected-accounts-list-item/connected-accounts-list-item.component.js, repos/metamask-extension/ui/components/app/assets/defi-list/defi-list.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance/account-group-balance.tsx, repos/metamask-extension/ui/components/app/assets/account-group-balance-change/account-group-balance-change.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/multiple-alert-modal/multiple-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/inline-alert/inline-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/general-alert/general-alert.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/confirm-alert-modal/confirm-alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-provider/alert-provider.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.stories.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/components/app/alert-system/alert-modal/alert-modal.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/confirmation/components/confirmation-network-switch/confirmation-network-switch.js, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/custom-amount/custom-amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/recipient-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/network-filter/network-filter.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-input/confusable-recipient-name.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/recipient-filter-input/recipient-filter-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/hex-data/hex-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount-recipient/amount-recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount-recipient/amount-recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/transactions/nested-transaction-tag/nested-transaction-tag.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-filter-input/asset-filter-input.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/total-row/total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/total-row/total-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/asset-list/asset-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/send/amount/amount.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/pay-with-row/pay-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/rows/required-tokens-row/required-tokens-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/info/custom-amount-info/custom-amount-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/developer/developer-button/developer-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/title/title.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/smart-account-tab.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/dataTree.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/scroll-to-bottom/scroll-to-bottom.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/scroll-to-bottom/scroll-to-bottom.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/nav/nav.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header-info.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/wallet-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/dapp-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/dapp-initiated-header.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/header/advanced-details-button.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-agreement.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/footer.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/origin-throttle-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/blockaid-loading-indicator/blockaid-loading-indicator.tsx, repos/metamask-extension/ui/pages/confirmations/components/advanced-gas-fee-popover/advanced-gas-fee-defaults/advanced-gas-fee-defaults.js, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-row/transaction-details-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-status-row/transaction-details-status-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-paid-with-row/transaction-details-paid-with-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-date-row/transaction-details-date-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-summary/transaction-details-summary.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details-hero/transaction-details-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/activity/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/asset/asset.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/send-hero/send-hero.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/pages/confirmations/components/UI/recipient/recipient.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-tooltip.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/gator-permissions/components/permission-list-item.tsx, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/pages/review-permissions-page/site-cell/site-cell-connection-list-item.js, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-change/percentage-change.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/price/percentage-and-amount-change/percentage-and-amount-change.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/custom-networks/custom-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/additional-networks-info/additional-networks-info.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/multichain/network-manager/components/default-networks/default-networks.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/confirm-turn-on-backup-and-sync-modal/confirm-turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/multichain-accounts/intro-modal/multichain-account-intro-modal.component.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/modals/identity/turn-on-backup-and-sync-modal/turn-on-backup-and-sync-modal.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/index.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/value-double.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/section.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/date.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/expandable-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/address.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/address.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/currency.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/text.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nfts-tab/nfts-tab.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-options/nft-options.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/url.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-row.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-grid/nft-grid.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-information-frame.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-detail-description.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-details.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-details/nft-full-image.tsx, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/toggle-ipfs-modal.js, repos/metamask-extension/ui/components/app/assets/nfts/nft-default-image/nft-default-image.tsx, repos/metamask-extension/ui/components/app/assets/defi-list/cells/defi-error-message.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/sort-control/sort-control.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/sort-control/sort-control.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/network-filter/network-filter.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/cells/generic-asset-cell-layout.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/components/app/assets/asset-list/asset-list-control-bar/asset-list-control-bar.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/snaps/snaps-section/snaps-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/smart-account-tab/account-network/account-network.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/typed-sign-data-v1/typedSignDataV1.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/typed-sign-data-v1/typedSignDataV1.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/typed-sign-data/typedSignData.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/row/typed-sign-data/typedSignData.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/transaction-flow-section.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/token-transfer/token-transfer.stories.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/personal-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/native-transfer/native-transfer.stories.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/nft-token-transfer/nft-token-transfer.stories.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-footer-coverage-indicator.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/footer/shield-footer-coverage-indicator/shield-footer-coverage-indicator.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/content/content.tsx, repos/metamask-extension/ui/components/multichain/pages/page/components/footer/footer.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/alert-row/alert-row.tsx, repos/metamask-extension/ui/components/app/confirm/info/row/alert-row/alert-row.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/components/app/import-token/network-filter-import-token/network-filter-dropdown/network-filter-drop-down-item/index.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/static-simulation/static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/send-heading/send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/selected-gas-fee-token/selected-gas-fee-token.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/transaction-data/transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/transaction-data/transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/transaction-data/transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/transaction-data/transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/nft-send-heading/nft-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/network-row/network-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-row/gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-toast/gas-fee-token-toast.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-list-item/gas-fee-token-list-item.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-icon/gas-fee-token-icon.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-icon/gas-fee-token-icon.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/native-send-heading/native-send-heading.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fee-token-modal/gas-fee-token-modal.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/gas-fees-details/gas-fees-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/confirm-loader/confirm-loader.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/batched-approval-function/batched-approval-function.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/personal-sign/siwe-sign/siwe-sign.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/revoke-set-approval-for-all-static-simulation/revoke-set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/revoke-set-approval-for-all-static-simulation/revoke-set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/revoke-set-approval-for-all-static-simulation/revoke-set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/revoke-set-approval-for-all-static-simulation/revoke-set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/set-approval-for-all-info/set-approval-for-all-static-simulation/set-approval-for-all-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/batch/nested-transaction-data/nested-transaction-data.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/revoke-static-simulation/revoke-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/revoke-static-simulation/revoke-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/revoke-static-simulation/revoke-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/revoke-static-simulation/revoke-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/approve/approve-static-simulation/approve-static-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/shared/edit-gas-fees-row/edit-gas-fees-row.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/native-value-display/native-value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/value-display/value-display.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/permit-simulation/permit-simulation.tsx, repos/metamask-extension/ui/pages/confirmations/components/confirm/info/typed-sign/typed-sign-v4-simulation/permit-simulation/permit-simulation.tsx</t>
   </si>
   <si>
     <t>BannerTip</t>
@@ -397,9 +400,6 @@
     <t>repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx</t>
   </si>
   <si>
-    <t>repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/reset-password-modal.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/unlock-page/unlock-page.component.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/srp-input-form/index.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/snap-account-redirect.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/snap-account-redirect.tsx, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/settings/settings.component.js, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/snap-account-card.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/remove-snap-account/remove-snap-account.tsx, repos/metamask-extension/ui/pages/permissions-connect/permissions-connect.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings.tsx, repos/metamask-extension/ui/pages/permissions-connect/permissions-connect.stories.js, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-flow.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-flow.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-types.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/notifications-settings/notifications-settings-allow-notifications.tsx, repos/metamask-extension/ui/pages/nonevm-balance-check/index.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.stories.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.stories.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details.stories.tsx, repos/metamask-extension/ui/pages/notifications/notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-placeholder.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-read-all-button.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-item.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-turn-on-notifications.tsx, repos/metamask-extension/ui/pages/notifications/notifications-list-item.stories.tsx, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/keychains/restore-vault.js, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/create-password-form/create-password-form.tsx, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/home/home.component.js, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/error-page/error-page.component.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/deep-link/deep-link.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/create-snap-account/create-snap-account.tsx, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/connected-accounts/connected-accounts.component.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/confirm-add-suggested-nft/confirm-add-suggested-nft.js, repos/metamask-extension/ui/pages/swaps/import-token/import-token.js, repos/metamask-extension/ui/pages/snap-account-redirect/components/url-display-box.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-message.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snap-account-redirect/components/snap-account-redirect-context.tsx, repos/metamask-extension/ui/pages/snaps/snap-view/snap-view.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snaps-list/snap-list.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/snaps/snap-view/snap-settings.js, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-animation.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/smart-transactions/smart-transaction-status-page/smart-transaction-status-page.tsx, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/settings-tab/settings-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/security-tab/security-tab.component.js, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/sentry-test.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-toggle-row-component.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/developer-options-tab.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/deprecated-network-modal/DeprecatedNetworkModal.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/developer-options-tab/backup-and-sync.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/contact-networks.tsx, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/settings/advanced-tab/advanced-tab.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/redirect/permissions-redirect.component.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/choose-account/choose-account.js, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/permissions-connect/connect-page/connect-page.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome-login.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-options.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/login-error-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/welcome/welcome.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/reveal-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/recovery-phrase-chips.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/review-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-srp-modal.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/recovery-phrase/confirm-recovery-phrase.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/privacy-settings/privacy-settings.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/metametrics/metametrics.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/onboarding-app-header/onboarding-app-header.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/onboarding-flow/create-password/create-password.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/download-app/download-app.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-not-found/account-not-found.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/creation-successful/creation-successful.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/onboarding-flow/account-exist/account-exist.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-body/notification-details-body.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-footer/notification-details-footer.tsx, repos/metamask-extension/ui/pages/notification-details/notification-details-footer/notification-details-footer.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/wallet-details-page/wallet-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-accounts-connect-page/multichain-accounts-connect-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/multichain-account-details-page/multichain-account-details-page.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multichain-accounts/account-list/account-list.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/multi-srp/import-srp/import-srp.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-list.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/defi/components/defi-details-page.tsx, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/create-account/connect-hardware/select-hardware.js, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/send/send-inner.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/confirmation.js, repos/metamask-extension/ui/pages/confirmations/confirmation/confirmation.js, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/tron-daily-resources.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/asset-page.tsx, repos/metamask-extension/ui/pages/asset/components/token-buttons.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/asset/components/asset-market-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-details.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/segment.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/segment.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/transaction-detail-row.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/hollow-circle.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/pulsing-circle.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/pulsing-circle.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/segment.stories.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-list.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-description.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-activity-item-tx-segments.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-activity-item-tx-segments.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-explorer-links.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-list.stories.tsx, repos/metamask-extension/ui/pages/bridge/transaction-details/bridge-step-list.stories.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/prepare-bridge-page.tsx, repos/metamask-extension/ui/pages/bridge/prepare/bridge-transaction-settings-modal.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/bridge/layout/tooltip.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/pages/bridge/awaiting-signatures/awaiting-signatures.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle/smart-contract-account-toggle.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/smart-contract-account-toggle-section/smart-contract-account-toggle-section.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-srp-backup/multichain-srp-backup.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-private-key-list/multichain-private-key-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-rows-list/multichain-address-rows-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-address-row/multichain-address-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-site-cell/multichain-site-cell.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-accounts-tree/multichain-accounts-tree.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu/multichain-account-menu.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-menu-items/multichain-account-menu-items.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-edit-modal/multichain-account-edit-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-list/multichain-account-list.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/edit-account-name-modal/edit-account-name-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/multichain-account-cell/multichain-account-cell.stories.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/add-multichain-account/add-multichain-account.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-show-srp-row/account-show-srp-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-remove-modal/account-remove-modal.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/multichain-accounts/account-details-row/account-details-row.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/qr-code-view/qr-code-view.tsx, repos/metamask-extension/ui/components/ui/origin-pill/origin-pill.tsx, repos/metamask-extension/ui/components/ui/metafox-logo/metafox-logo.component.js, repos/metamask-extension/ui/components/ui/logo/logo.stories.js, repos/metamask-extension/ui/components/ui/loading-screen/loading-screen.component.js, repos/metamask-extension/ui/components/ui/loading-screen/loading-screen.component.js, repos/metamask-extension/ui/components/ui/loading-screen/loading-screen.component.js, repos/metamask-extension/ui/components/ui/loading-indicator/loading-indicator.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/form-field/form-field.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/editable-label/editable-label.js, repos/metamask-extension/ui/components/ui/export-text-container/export-text-container.component.js, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/delineator/delineator.tsx, repos/metamask-extension/ui/components/ui/currency-display/currency-display.component.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/callout/callout.stories.js, repos/metamask-extension/ui/components/ui/aggregated-balance/aggregated-balance.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/multichain/toast/toast.tsx, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/ui/account-list/account-list.js, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/token-list-item.tsx, repos/metamask-extension/ui/components/multichain/token-list-item/stakeable-link.tsx, repos/metamask-extension/ui/components/multichain/receive-modal/receive-modal.js, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/notifications-tag-counter/notifications-tag-counter.tsx, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/product-tour-popover/product-tour-popover.js, repos/metamask-extension/ui/components/multichain/permissions-header/permissions-header.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-type/notifications-settings-type.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-box/notifications-settings-box.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notifications-settings-account/notifications-settings-account.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-title/notification-detail-title.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-snap/notification-list-item-snap.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item-icon/notification-list-item-icon.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-list-item/notification-list-item.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-nft/notification-detail-nft.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-nft/notification-detail-nft.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-copy-button/notification-detail-copy-button.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-collection/notification-detail-collection.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail-network-fee/notification-detail-network-fee.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/notification-detail/notification-detail.tsx, repos/metamask-extension/ui/components/multichain/network-manager/network-tabs.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/nft-item/nft-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/rpc-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-menu/network-list-menu.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item/network-list-item.tsx, repos/metamask-extension/ui/components/multichain/network-list-item-menu/network-list-item-menu.js, repos/metamask-extension/ui/components/multichain/network-filter-menu/index.tsx, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-nfts-modal/import-nfts-modal.js, repos/metamask-extension/ui/components/multichain/import-account/import-account.js, repos/metamask-extension/ui/components/multichain/import-account/bottom-buttons.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal-confirm.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/import-tokens-modal/import-tokens-modal.js, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/funding-method-modal/funding-method-item.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/edit-accounts-modal.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-new-account-option.tsx, repos/metamask-extension/ui/components/multichain/edit-accounts-modal/add-account.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/dropdown-editor/dropdown-editor.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/domain-input-resolution-cell/domain-input-resolution-cell.tsx, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/edit-networks-modal/edit-networks-modal.js, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-solana-account-modal/create-solana-account-modal.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/create-account/create-account.tsx, repos/metamask-extension/ui/components/multichain/connected-site-menu/connected-site-menu.js, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/connected-site-popover/connected-site-popover.tsx, repos/metamask-extension/ui/components/multichain/carousel/carousel.tsx, repos/metamask-extension/ui/components/multichain/carousel/carousel.tsx, repos/metamask-extension/ui/components/multichain/app-header/multichain-meta-fox-logo.js, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/avatar-group/avatar-group.tsx, repos/metamask-extension/ui/components/multichain/connect-accounts-modal/connect-accounts-modal-list.tsx, repos/metamask-extension/ui/components/multichain/app-header/app-header.js, repos/metamask-extension/ui/components/multichain/app-header/app-header-container.tsx, repos/metamask-extension/ui/components/multichain/badge-status/badge-status.tsx, repos/metamask-extension/ui/components/multichain/badge-status/badge-status.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.stories.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.stories.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.stories.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-list-item/address-list-item.tsx, repos/metamask-extension/ui/components/multichain/address-copy-button/address-copy-button.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/account-picker/account-picker.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.js, repos/metamask-extension/ui/components/multichain/activity-list-item/activity-list-item.stories.js, repos/metamask-extension/ui/components/multichain/account-overview/account-overview-unknown.tsx, repos/metamask-extension/ui/components/multichain/account-overview/account-overview-unknown.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-menu/account-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/hidden-account-list.js, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-list-menu/account-list-menu.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-network-indicator/account-network-indicator.tsx, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-list-item/account-list-item.js, repos/metamask-extension/ui/components/multichain/account-details/account-details.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-key.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-authenticate.js, repos/metamask-extension/ui/components/app/wallet-overview/coin-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview.tsx, repos/metamask-extension/ui/components/app/wallet-overview/coin-buttons.tsx, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/multichain/account-details/account-details-display.js, repos/metamask-extension/ui/components/app/wallet-overview/aggregated-percentage-overview-cross-chains.tsx, repos/metamask-extension/ui/components/app/update-modal/update-modal.tsx, repos/metamask-extension/ui/components/app/transaction-list-item-details/transaction-list-item-details.component.js, repos/metamask-extension/ui/components/app/transaction-list/unified-transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/transaction-list-item.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list/transaction-list.component.js, repos/metamask-extension/ui/components/app/transaction-list-item/smart-transaction-list-item.component.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/terms-of-use-popup/terms-of-use-popup.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.js, repos/metamask-extension/ui/components/app/tab-bar/tab-bar.js, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-input-import/srp-input-import.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/srp-details-modal/srp-details-modal.tsx, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/recovery-phrase-reminder/recovery-phrase-reminder.js, repos/metamask-extension/ui/components/app/permissions-connect-permission-list/permissions-connect-permission-list.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-connect-header/permission-connect-header.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell-status.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permission-cell/permission-cell.js, repos/metamask-extension/ui/components/app/permissions-connect-footer/permissions-connect-footer.component.js, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-outdated-modal/password-outdated-modal.tsx, repos/metamask-extension/ui/components/app/password-form/password-form.tsx, repos/metamask-extension/ui/components/app/permission-page-container/permission-page-container.component.js, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-list-item/multichain-bridge-transaction-list-item.tsx, repos/metamask-extension/ui/components/app/name/name.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multi-rpc-edit-modal/multi-rpc-edit-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-bridge-transaction-details-modal/multichain-bridge-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/multichain-transaction-details-modal/multichain-transaction-details-modal.tsx, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/hold-to-reveal-button/hold-to-reveal-button.js, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/download-mobile-modal/download-mobile-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/data-deletion-error-modal/data-deletion-error-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/connections-removed-modal/connections-removed-modal.tsx, repos/metamask-extension/ui/components/app/currency-input/currency-input.js, repos/metamask-extension/ui/components/app/currency-input/currency-input.js, repos/metamask-extension/ui/components/app/currency-input/currency-input.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/connected-sites-list/connected-snaps.js, repos/metamask-extension/ui/components/app/configure-snap-popup/configure-snap-popup.tsx, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/connected-accounts-permissions/connected-accounts-permissions.js, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/clear-metametrics-data/clear-metametrics-data.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/components/app/basic-configuration-modal/basic-configuration-modal.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/delete-metametrics-data-button/delete-metametrics-data-button.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/reveal-srp-list/reveal-srp-list.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/metametrics-toggle/metametrics-toggle.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/networks-tab/networks-form/networks-form.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/add-contact/add-contact.component.js, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/security-tab/change-password/change-password-warning.tsx, repos/metamask-extension/ui/pages/settings/contact-list-tab/view-contact/view-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/settings/contact-list-tab/edit-contact/edit-contact.component.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snaps-connect/snaps-connect.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-update/snap-update.js, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/snap/snap.tsx, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/permissions-connect/snaps/snap-install/snap-install.js, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/notifications/notification-components/feature-announcement/feature-announcement.tsx, repos/metamask-extension/ui/pages/confirmations/confirmation/stories/util.js, repos/metamask-extension/ui/pages/confirmations/confirmation/stories/util.js, repos/metamask-extension/ui/pages/confirmations/confirmation/stories/util.js, repos/metamask-extension/ui/pages/confirmations/components/smart-contract-with-logo/smart-contract-with-logo.tsx, repos/metamask-extension/ui/pages/confirmations/components/smart-transactions-banner-alert/smart-transactions-banner-alert.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/simulation-details.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-list.tsx, repos/metamask-extension/ui/pages/confirmations/components/simulation-details/balance-change-list.tsx, repo